<commit_message>
chore: update funding tracker
</commit_message>
<xml_diff>
--- a/近期融资公司追踪.xlsx
+++ b/近期融资公司追踪.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="R5f166eea3e264e13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="Rd5906e8889d64ccc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="R6eba3617dbf84fd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="Rbe8b19f2661f47e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="Rf27b78d9708a4cc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="R047508d4d4c541f7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -418,61 +418,63 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
-        <x:v>中科世通亨奇</x:v>
+        <x:v>中科国晟</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>智能决策基础设施 / 空间计算</x:v>
+        <x:v>燃气轮机 / 动力装备</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
-        <x:v>46272.333333333336</x:v>
+        <x:v>46283.333333333336</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>近5亿元人民币</x:v>
+        <x:v>6亿元人民币</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>B 系列融资</x:v>
+        <x:v>C轮</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G5" s="14"/>
+      <x:c r="G5" s="14" t="n">
+        <x:v>60000</x:v>
+      </x:c>
       <x:c r="H5" s="12" t="str">
-        <x:v>证券时报 / 同花顺财经</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I5" s="16" t="str">
-        <x:v>https://m.10jqka.com.cn/20260907/c679650478.shtml</x:v>
+        <x:v>https://news.pedaily.cn/202609/569246.shtml</x:v>
       </x:c>
       <x:c r="J5" s="15" t="n">
-        <x:v>46272.748611111114</x:v>
+        <x:v>46283.534479166665</x:v>
       </x:c>
       <x:c r="K5" s="12" t="str">
         <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L5" s="12" t="str">
-        <x:v>中科世通亨奇面向智能决策基础设施、空间计算与复杂系统仿真场景，打造 AOS 时空智能基础设施及世通灵境产品体系。公司服务城市治理、应急安全、低空经济、机器人和国防军工等高复杂度决策场景，强调三维空间、实时数据和智能推演能力融合。</x:v>
+        <x:v>中科国晟动力科技有限公司专注轻型燃气轮机及相关动力装备的研发、制造和服务。公司围绕燃气轮机核心技术、试验验证、批量生产与全生命周期服务建设能力，面向分布式能源、工业动力和特种装备等应用场景。</x:v>
       </x:c>
       <x:c r="M5" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.qdzkgs.com/</x:v>
       </x:c>
       <x:c r="N5" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>商务邮箱：scb@qdzkgs.com；官网公开电话：18678960108；官网： https://www.qdzkgs.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
-        <x:v>日耀光电</x:v>
+        <x:v>铬莱铂</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>光伏 / 钙钛矿材料</x:v>
+        <x:v>金属3D打印 / 增材制造</x:v>
       </x:c>
       <x:c r="C6" s="13" t="n">
-        <x:v>46269.333333333336</x:v>
+        <x:v>46283.333333333336</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>数千万元人民币</x:v>
+        <x:v>近2亿元人民币</x:v>
       </x:c>
       <x:c r="E6" s="12" t="str">
-        <x:v>Pre-A 轮</x:v>
+        <x:v>A轮</x:v>
       </x:c>
       <x:c r="F6" s="12" t="str">
         <x:v>CNY</x:v>
@@ -482,39 +484,39 @@
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I6" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%97%A5%E8%80%80%E5%85%89%E7%94%B5%20%E6%95%B0%E5%8D%83%E4%B8%87%E5%85%83%20Pre-A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202609/569242.shtml</x:v>
       </x:c>
       <x:c r="J6" s="15" t="n">
-        <x:v>46272.748611111114</x:v>
+        <x:v>46283.534479166665</x:v>
       </x:c>
       <x:c r="K6" s="12" t="str">
-        <x:v>媒体核验；官网待交叉确认</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L6" s="12" t="str">
-        <x:v>日耀光电聚焦钙钛矿光伏材料与器件研发，围绕新型太阳能电池材料、工艺和应用推进产业化。公司所处赛道面向高效率、低成本光伏技术迭代，可服务下一代光伏组件和分布式能源应用。</x:v>
+        <x:v>铬莱铂是一家金属增材制造企业，围绕 SLM 金属 3D 打印设备、打印服务和智能化工厂解决方案开展业务。公司布局金属 3D 打印装备生产基地与服务基地，服务航空航天、工业制造和复杂金属零部件的快速制造需求。</x:v>
       </x:c>
       <x:c r="M6" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.glb3d.cn/</x:v>
       </x:c>
       <x:c r="N6" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官网公开电话：13856183190；官网联系页：https://www.glb3d.cn/</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
-        <x:v>记忆张量</x:v>
+        <x:v>上海斐睿科思</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>AI 记忆基础设施</x:v>
+        <x:v>生命科学具身智能 / 数据基础设施</x:v>
       </x:c>
       <x:c r="C7" s="13" t="n">
-        <x:v>46269.333333333336</x:v>
+        <x:v>46283.333333333336</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>数百万元人民币</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
-        <x:v>Pre-A+ 轮</x:v>
+        <x:v>首轮战略投资</x:v>
       </x:c>
       <x:c r="F7" s="12" t="str">
         <x:v>CNY</x:v>
@@ -524,39 +526,39 @@
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I7" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E8%AE%B0%E5%BF%86%E5%BC%A0%E9%87%8F%20Pre-A%2B%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202609/569241.shtml</x:v>
       </x:c>
       <x:c r="J7" s="15" t="n">
-        <x:v>46272.748611111114</x:v>
+        <x:v>46283.534479166665</x:v>
       </x:c>
       <x:c r="K7" s="12" t="str">
-        <x:v>媒体与官网交叉核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L7" s="12" t="str">
-        <x:v>记忆张量专注 AI 记忆基础设施，推进 MemOS 等面向智能体和大模型应用的长期记忆系统。公司尝试把记忆管理、上下文组织和个性化知识沉淀做成基础层能力，服务企业级 AI Agent 与持续学习场景。</x:v>
+        <x:v>上海斐睿科思聚焦生命科学领域的具身智能数据基础设施，建设数据采集与训练实验室、机器人系统和跨设备适配能力。公司希望用机器人与 Physical AI 支持生命科学实验数据生产、训练和科研流程自动化。</x:v>
       </x:c>
       <x:c r="M7" s="12" t="str">
-        <x:v>https://www.memtensor.cn/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N7" s="12" t="str">
-        <x:v>官网提供产品介绍与在线访问入口；未找到可交叉确认的公开商务电话或邮箱。</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
-        <x:v>中科昊芯</x:v>
+        <x:v>弧光量子</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>DSP 芯片 / 工业控制</x:v>
+        <x:v>量子计算 / 量子软件</x:v>
       </x:c>
       <x:c r="C8" s="13" t="n">
-        <x:v>46269.333333333336</x:v>
+        <x:v>46283.333333333336</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>超亿元人民币</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
-        <x:v>B 轮</x:v>
+        <x:v>战略融资</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
         <x:v>CNY</x:v>
@@ -566,39 +568,39 @@
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I8" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E4%B8%AD%E7%A7%91%E6%98%8A%E8%8A%AF%20B%E8%BD%AE%20%E8%9E%8D%E8%B5%84%20%E6%82%A6%E6%B9%96%E8%B5%84%E6%9C%AC&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202609/569239.shtml</x:v>
       </x:c>
       <x:c r="J8" s="15" t="n">
-        <x:v>46272.748611111114</x:v>
+        <x:v>46283.534479166665</x:v>
       </x:c>
       <x:c r="K8" s="12" t="str">
-        <x:v>媒体与官网交叉核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L8" s="12" t="str">
-        <x:v>中科昊芯从事高性能 DSP 芯片及嵌入式处理器研发，产品面向工业控制、电力电子、新能源、机器人和高端装备等场景。公司围绕国产实时控制芯片、开发工具链和生态适配推进产业化落地。</x:v>
+        <x:v>弧光量子专注量子计算软件与量子应用研发，推进量子计算与人工智能的融合。公司围绕分布式芯片、新型测控架构和量子软件能力开展研发，面向量子计算产业化和高性能计算应用场景。</x:v>
       </x:c>
       <x:c r="M8" s="12" t="str">
-        <x:v>https://www.haawking.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N8" s="12" t="str">
-        <x:v>官网联系页：https://www.haawking.com/contact.html</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
-        <x:v>追梦空天</x:v>
+        <x:v>枢途科技</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>航空航天 / 混动 eVTOL</x:v>
+        <x:v>触觉技术 / 具身智能数据基础设施</x:v>
       </x:c>
       <x:c r="C9" s="13" t="n">
-        <x:v>46268.333333333336</x:v>
+        <x:v>46283.333333333336</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
         <x:v>近亿元人民币</x:v>
       </x:c>
       <x:c r="E9" s="12" t="str">
-        <x:v>天使轮</x:v>
+        <x:v>Pre-A轮</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str">
         <x:v>CNY</x:v>
@@ -608,100 +610,102 @@
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I9" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E8%BF%BD%E6%A2%A6%E7%A9%BA%E5%A4%A9%20%E8%BF%91%E4%BA%BF%E5%85%83%20%E5%A4%A9%E4%BD%BF%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202609/569233.shtml</x:v>
       </x:c>
       <x:c r="J9" s="15" t="n">
-        <x:v>46272.748611111114</x:v>
+        <x:v>46283.534479166665</x:v>
       </x:c>
       <x:c r="K9" s="12" t="str">
-        <x:v>媒体核验；官网待交叉确认</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L9" s="12" t="str">
-        <x:v>追梦空天聚焦混动 eVTOL 与低空出行飞行器研发，推进 DF3000 等长航程、高载荷航空器产品。公司面向低空物流、通勤出行、应急救援和特种作业等场景探索混合动力飞行平台商业化。</x:v>
+        <x:v>枢途科技聚焦触觉技术和具身智能数据基础设施，研发 SynaTac 等触觉技术与产品，并提供人类行为数据采集和交付能力。公司面向机器人接触智能、生命科学和具身智能训练场景，建设从数据生产到机器人应用的技术链路。</x:v>
       </x:c>
       <x:c r="M9" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.synapath.com/</x:v>
       </x:c>
       <x:c r="N9" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官网已核验；未检索到公开商务邮箱或电话，可通过官网联系入口咨询。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="12" t="str">
-        <x:v>优宝特</x:v>
+        <x:v>奕行智能</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>智能机器人 / 工业自动化</x:v>
+        <x:v>RISC-V / AI芯片</x:v>
       </x:c>
       <x:c r="C10" s="13" t="n">
-        <x:v>46268.333333333336</x:v>
+        <x:v>46283.333333333336</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>20亿元人民币</x:v>
       </x:c>
       <x:c r="E10" s="12" t="str">
-        <x:v>A+ 轮</x:v>
+        <x:v>新一轮融资</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G10" s="14"/>
+      <x:c r="G10" s="14" t="n">
+        <x:v>200000</x:v>
+      </x:c>
       <x:c r="H10" s="12" t="str">
-        <x:v>科创板日报</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I10" s="16" t="str">
-        <x:v>https://www.chinastarmarket.cn/detail/2473458</x:v>
+        <x:v>https://news.pedaily.cn/202609/569236.shtml</x:v>
       </x:c>
       <x:c r="J10" s="15" t="n">
-        <x:v>46272.748611111114</x:v>
+        <x:v>46283.534479166665</x:v>
       </x:c>
       <x:c r="K10" s="12" t="str">
-        <x:v>媒体与官网交叉核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L10" s="12" t="str">
-        <x:v>优宝特是智能机器人与工业自动化企业，产品覆盖冲压自动化、焊装自动化、智能仓储物流及移动机器人等方向。公司面向汽车、家电、工程机械和智能制造场景提供机器人本体、系统集成与产线自动化解决方案。</x:v>
+        <x:v>奕行智能专注 RISC-V 处理器、AI 算力芯片及相关软硬件系统研发。公司围绕自主指令集架构、智能计算和芯片生态建设产品能力，面向数据中心、边缘计算和行业智能化场景推进落地。</x:v>
       </x:c>
       <x:c r="M10" s="12" t="str">
-        <x:v>https://www.yobotics.cn/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N10" s="12" t="str">
-        <x:v>官网联系页：https://www.yobotics.cn/</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
-        <x:v>Violoop（本惟无界）</x:v>
+        <x:v>中科世通亨奇</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>AI 眼镜 / 消费电子</x:v>
+        <x:v>智能决策基础设施 / 空间计算</x:v>
       </x:c>
       <x:c r="C11" s="13" t="n">
-        <x:v>46266.333333333336</x:v>
+        <x:v>46272.333333333336</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
-        <x:v>亿元级人民币</x:v>
+        <x:v>近5亿元人民币</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
-        <x:v>Pre-A 轮</x:v>
+        <x:v>B 系列融资</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G11" s="14"/>
       <x:c r="H11" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>证券时报 / 同花顺财经</x:v>
       </x:c>
       <x:c r="I11" s="16" t="str">
-        <x:v>https://news.google.com/search?q=Violoop%20%E6%9C%AC%E6%83%9F%E6%97%A0%E7%95%8C%20%E4%BA%BF%E5%85%83%E7%BA%A7%20Pre-A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://m.10jqka.com.cn/20260907/c679650478.shtml</x:v>
       </x:c>
       <x:c r="J11" s="15" t="n">
         <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K11" s="12" t="str">
-        <x:v>媒体核验；官网待交叉确认</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L11" s="12" t="str">
-        <x:v>Violoop（本惟无界）面向 AI 眼镜和下一代可穿戴计算终端研发硬件与交互系统。公司围绕多模态感知、端侧智能和轻量化消费电子产品形态，探索智能眼镜在日常助理、拍摄记录和空间交互中的应用。</x:v>
+        <x:v>中科世通亨奇面向智能决策基础设施、空间计算与复杂系统仿真场景，打造 AOS 时空智能基础设施及世通灵境产品体系。公司服务城市治理、应急安全、低空经济、机器人和国防军工等高复杂度决策场景，强调三维空间、实时数据和智能推演能力融合。</x:v>
       </x:c>
       <x:c r="M11" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -712,38 +716,38 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>芯光界</x:v>
+        <x:v>日耀光电</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>光互连 / 硅光通信</x:v>
+        <x:v>光伏 / 钙钛矿材料</x:v>
       </x:c>
       <x:c r="C12" s="13" t="n">
-        <x:v>46266.333333333336</x:v>
+        <x:v>46269.333333333336</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
-        <x:v>天使+轮</x:v>
+        <x:v>Pre-A 轮</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G12" s="14"/>
       <x:c r="H12" s="12" t="str">
-        <x:v>中国证券报·中证网</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I12" s="16" t="str">
-        <x:v>https://www.cs.com.cn/tzjj/01/2026/09/02/detail_2026090210036492.html</x:v>
+        <x:v>https://news.google.com/search?q=%E6%97%A5%E8%80%80%E5%85%89%E7%94%B5%20%E6%95%B0%E5%8D%83%E4%B8%87%E5%85%83%20Pre-A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J12" s="15" t="n">
-        <x:v>46272.77361111111</x:v>
+        <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K12" s="12" t="str">
         <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L12" s="12" t="str">
-        <x:v>芯光界面向 AI 算力集群和高速通信场景研发硅光互连与光电融合产品。公司聚焦低功耗、高带宽、可规模化部署的光互连方案，服务数据中心、智算中心和下一代网络基础设施。</x:v>
+        <x:v>日耀光电聚焦钙钛矿光伏材料与器件研发，围绕新型太阳能电池材料、工艺和应用推进产业化。公司所处赛道面向高效率、低成本光伏技术迭代，可服务下一代光伏组件和分布式能源应用。</x:v>
       </x:c>
       <x:c r="M12" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -754,19 +758,19 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="str">
-        <x:v>先博生物</x:v>
+        <x:v>记忆张量</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
-        <x:v>创新药 / 细胞治疗</x:v>
+        <x:v>AI 记忆基础设施</x:v>
       </x:c>
       <x:c r="C13" s="13" t="n">
-        <x:v>46265.333333333336</x:v>
+        <x:v>46269.333333333336</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>近4亿元人民币</x:v>
+        <x:v>未披露</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>Pre-A+ 轮</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
         <x:v>CNY</x:v>
@@ -776,7 +780,7 @@
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I13" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%85%88%E5%8D%9A%E7%94%9F%E7%89%A9%20%E8%BF%914%E4%BA%BF%E5%85%83%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E8%AE%B0%E5%BF%86%E5%BC%A0%E9%87%8F%20Pre-A%2B%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J13" s="15" t="n">
         <x:v>46272.748611111114</x:v>
@@ -785,27 +789,27 @@
         <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L13" s="12" t="str">
-        <x:v>先博生物（Simnova Bio）是一家创新药和细胞治疗公司，重点推进实体瘤及免疫相关疾病方向的候选产品研发。公司围绕细胞治疗、基因工程和转化医学平台建设管线，服务临床未满足需求。</x:v>
+        <x:v>记忆张量专注 AI 记忆基础设施，推进 MemOS 等面向智能体和大模型应用的长期记忆系统。公司尝试把记忆管理、上下文组织和个性化知识沉淀做成基础层能力，服务企业级 AI Agent 与持续学习场景。</x:v>
       </x:c>
       <x:c r="M13" s="12" t="str">
-        <x:v>https://www.simnovabio.com/</x:v>
+        <x:v>https://www.memtensor.cn/</x:v>
       </x:c>
       <x:c r="N13" s="12" t="str">
-        <x:v>官网联系页：https://www.simnovabio.com/cn/contact-us</x:v>
+        <x:v>官网提供产品介绍与在线访问入口；未找到可交叉确认的公开商务电话或邮箱。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="12" t="str">
-        <x:v>沐创集成电路</x:v>
+        <x:v>中科昊芯</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
-        <x:v>智能网卡 / 高速互联芯片</x:v>
+        <x:v>DSP 芯片 / 工业控制</x:v>
       </x:c>
       <x:c r="C14" s="13" t="n">
-        <x:v>46264.333333333336</x:v>
+        <x:v>46269.333333333336</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>未披露</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
         <x:v>B 轮</x:v>
@@ -815,145 +819,145 @@
       </x:c>
       <x:c r="G14" s="14"/>
       <x:c r="H14" s="12" t="str">
-        <x:v>园区世界投融资周报</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I14" s="16" t="str">
-        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
+        <x:v>https://news.google.com/search?q=%E4%B8%AD%E7%A7%91%E6%98%8A%E8%8A%AF%20B%E8%BD%AE%20%E8%9E%8D%E8%B5%84%20%E6%82%A6%E6%B9%96%E8%B5%84%E6%9C%AC&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J14" s="15" t="n">
-        <x:v>46272.77361111111</x:v>
+        <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K14" s="12" t="str">
         <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L14" s="12" t="str">
-        <x:v>沐创集成电路专注智能网卡、DPU 和高速互联芯片研发，面向数据中心、云计算和智算基础设施提供网络与数据处理芯片。公司产品服务高吞吐、低延迟的数据传输和计算卸载场景。</x:v>
+        <x:v>中科昊芯从事高性能 DSP 芯片及嵌入式处理器研发，产品面向工业控制、电力电子、新能源、机器人和高端装备等场景。公司围绕国产实时控制芯片、开发工具链和生态适配推进产业化落地。</x:v>
       </x:c>
       <x:c r="M14" s="12" t="str">
-        <x:v>https://www.mucse.com/</x:v>
+        <x:v>https://www.haawking.com/</x:v>
       </x:c>
       <x:c r="N14" s="12" t="str">
-        <x:v>官网联系页：https://www.mucse.com/contact.html</x:v>
+        <x:v>官网联系页：https://www.haawking.com/contact.html</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>研微半导体</x:v>
+        <x:v>追梦空天</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
-        <x:v>半导体设备 / 薄膜沉积</x:v>
+        <x:v>航空航天 / 混动 eVTOL</x:v>
       </x:c>
       <x:c r="C15" s="13" t="n">
-        <x:v>46264.333333333336</x:v>
+        <x:v>46268.333333333336</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>近15亿元人民币</x:v>
+        <x:v>近亿元人民币</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
-        <x:v>B 轮</x:v>
+        <x:v>天使轮</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G15" s="14"/>
       <x:c r="H15" s="12" t="str">
-        <x:v>园区世界投融资周报</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I15" s="16" t="str">
-        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
+        <x:v>https://news.google.com/search?q=%E8%BF%BD%E6%A2%A6%E7%A9%BA%E5%A4%A9%20%E8%BF%91%E4%BA%BF%E5%85%83%20%E5%A4%A9%E4%BD%BF%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J15" s="15" t="n">
-        <x:v>46272.77361111111</x:v>
+        <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K15" s="12" t="str">
-        <x:v>媒体与官网交叉核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L15" s="12" t="str">
-        <x:v>研微半导体聚焦半导体薄膜沉积设备和关键制程装备研发，服务集成电路、先进封装和泛半导体制造。公司围绕国产半导体设备替代、工艺适配和产线交付推进产业化。</x:v>
+        <x:v>追梦空天聚焦混动 eVTOL 与低空出行飞行器研发，推进 DF3000 等长航程、高载荷航空器产品。公司面向低空物流、通勤出行、应急救援和特种作业等场景探索混合动力飞行平台商业化。</x:v>
       </x:c>
       <x:c r="M15" s="12" t="str">
-        <x:v>https://www.psrsemi.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N15" s="12" t="str">
-        <x:v>官网联系页：https://www.psrsemi.com/</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
-        <x:v>迈步机器人</x:v>
+        <x:v>优宝特</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>康复机器人 / 外骨骼</x:v>
+        <x:v>智能机器人 / 工业自动化</x:v>
       </x:c>
       <x:c r="C16" s="13" t="n">
-        <x:v>46264.333333333336</x:v>
+        <x:v>46268.333333333336</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>近亿元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
-        <x:v>战略融资</x:v>
+        <x:v>A+ 轮</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G16" s="14"/>
       <x:c r="H16" s="12" t="str">
-        <x:v>园区世界投融资周报</x:v>
+        <x:v>科创板日报</x:v>
       </x:c>
       <x:c r="I16" s="16" t="str">
-        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
+        <x:v>https://www.chinastarmarket.cn/detail/2473458</x:v>
       </x:c>
       <x:c r="J16" s="15" t="n">
-        <x:v>46272.77361111111</x:v>
+        <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K16" s="12" t="str">
         <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L16" s="12" t="str">
-        <x:v>迈步机器人是一家康复机器人和外骨骼设备企业，产品覆盖下肢康复训练、步态训练和智能辅助行走等方向。公司面向医院、康复中心和家庭康复场景，结合机器人控制、传感和康复医学提升训练效率。</x:v>
+        <x:v>优宝特是智能机器人与工业自动化企业，产品覆盖冲压自动化、焊装自动化、智能仓储物流及移动机器人等方向。公司面向汽车、家电、工程机械和智能制造场景提供机器人本体、系统集成与产线自动化解决方案。</x:v>
       </x:c>
       <x:c r="M16" s="12" t="str">
-        <x:v>https://www.milebot.com/</x:v>
+        <x:v>https://www.yobotics.cn/</x:v>
       </x:c>
       <x:c r="N16" s="12" t="str">
-        <x:v>官网联系页：https://www.milebot.com/contact.html</x:v>
+        <x:v>官网联系页：https://www.yobotics.cn/</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
-        <x:v>屹艮科技</x:v>
+        <x:v>Violoop（本惟无界）</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>AI for Science / 电池设计自动化</x:v>
+        <x:v>AI 眼镜 / 消费电子</x:v>
       </x:c>
       <x:c r="C17" s="13" t="n">
-        <x:v>46264.333333333336</x:v>
+        <x:v>46266.333333333336</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
         <x:v>亿元级人民币</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
-        <x:v>战略融资</x:v>
+        <x:v>Pre-A 轮</x:v>
       </x:c>
       <x:c r="F17" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G17" s="14"/>
       <x:c r="H17" s="12" t="str">
-        <x:v>园区世界投融资周报</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I17" s="16" t="str">
-        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
+        <x:v>https://news.google.com/search?q=Violoop%20%E6%9C%AC%E6%83%9F%E6%97%A0%E7%95%8C%20%E4%BA%BF%E5%85%83%E7%BA%A7%20Pre-A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J17" s="15" t="n">
-        <x:v>46272.77361111111</x:v>
+        <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K17" s="12" t="str">
         <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L17" s="12" t="str">
-        <x:v>屹艮科技面向电池材料研发和电池设计自动化建设 AI for Science 平台，支持材料筛选、配方设计和性能预测。公司将机器学习、实验数据和多尺度仿真结合，服务新能源电池研发效率提升。</x:v>
+        <x:v>Violoop（本惟无界）面向 AI 眼镜和下一代可穿戴计算终端研发硬件与交互系统。公司围绕多模态感知、端侧智能和轻量化消费电子产品形态，探索智能眼镜在日常助理、拍摄记录和空间交互中的应用。</x:v>
       </x:c>
       <x:c r="M17" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -964,115 +968,113 @@
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
-        <x:v>中数睿智</x:v>
+        <x:v>芯光界</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
-        <x:v>大模型 / 企业 AI Agent</x:v>
+        <x:v>光互连 / 硅光通信</x:v>
       </x:c>
       <x:c r="C18" s="13" t="n">
-        <x:v>46264.333333333336</x:v>
+        <x:v>46266.333333333336</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
         <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
-        <x:v>战略融资</x:v>
+        <x:v>天使+轮</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G18" s="14"/>
       <x:c r="H18" s="12" t="str">
-        <x:v>园区世界投融资周报</x:v>
+        <x:v>中国证券报·中证网</x:v>
       </x:c>
       <x:c r="I18" s="16" t="str">
-        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
+        <x:v>https://www.cs.com.cn/tzjj/01/2026/09/02/detail_2026090210036492.html</x:v>
       </x:c>
       <x:c r="J18" s="15" t="n">
         <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K18" s="12" t="str">
-        <x:v>媒体与官网交叉核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L18" s="12" t="str">
-        <x:v>中数睿智聚焦企业级大模型和 AI Agent 应用，推出语思等面向行业知识、办公协同和智能决策的产品体系。公司服务政府、央国企和大型组织的数字化与智能化升级场景。</x:v>
+        <x:v>芯光界面向 AI 算力集群和高速通信场景研发硅光互连与光电融合产品。公司聚焦低功耗、高带宽、可规模化部署的光互连方案，服务数据中心、智算中心和下一代网络基础设施。</x:v>
       </x:c>
       <x:c r="M18" s="12" t="str">
-        <x:v>https://www.zhongshuruizhi.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N18" s="12" t="str">
-        <x:v>官网联系页：https://www.zhongshuruizhi.com/</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="12" t="str">
-        <x:v>星邑空间</x:v>
+        <x:v>先博生物</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
-        <x:v>商业航天 / 卫星测运控</x:v>
+        <x:v>创新药 / 细胞治疗</x:v>
       </x:c>
       <x:c r="C19" s="13" t="n">
-        <x:v>46264.333333333336</x:v>
+        <x:v>46265.333333333336</x:v>
       </x:c>
       <x:c r="D19" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>近4亿元人民币</x:v>
       </x:c>
       <x:c r="E19" s="12" t="str">
-        <x:v>A 轮增资扩股</x:v>
+        <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F19" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G19" s="14"/>
       <x:c r="H19" s="12" t="str">
-        <x:v>园区世界投融资周报</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I19" s="16" t="str">
-        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
+        <x:v>https://news.google.com/search?q=%E5%85%88%E5%8D%9A%E7%94%9F%E7%89%A9%20%E8%BF%914%E4%BA%BF%E5%85%83%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J19" s="15" t="n">
-        <x:v>46272.77361111111</x:v>
+        <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K19" s="12" t="str">
         <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L19" s="12" t="str">
-        <x:v>星邑空间从事商业航天测运控、卫星数据服务和空间信息基础设施建设，面向卫星运营、遥感应用和低轨星座服务提供能力。公司围绕地面站网络、测控调度和空间数据应用推进商业化。</x:v>
+        <x:v>先博生物（Simnova Bio）是一家创新药和细胞治疗公司，重点推进实体瘤及免疫相关疾病方向的候选产品研发。公司围绕细胞治疗、基因工程和转化医学平台建设管线，服务临床未满足需求。</x:v>
       </x:c>
       <x:c r="M19" s="12" t="str">
-        <x:v>https://www.xingyispace.com/</x:v>
+        <x:v>https://www.simnovabio.com/</x:v>
       </x:c>
       <x:c r="N19" s="12" t="str">
-        <x:v>官网联系页：https://www.xingyispace.com/</x:v>
+        <x:v>官网联系页：https://www.simnovabio.com/cn/contact-us</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="12" t="str">
-        <x:v>瞬适科技</x:v>
+        <x:v>沐创集成电路</x:v>
       </x:c>
       <x:c r="B20" s="12" t="str">
-        <x:v>具身智能 / 物理 AI 数据基础设施</x:v>
+        <x:v>智能网卡 / 高速互联芯片</x:v>
       </x:c>
       <x:c r="C20" s="13" t="n">
-        <x:v>46262.333333333336</x:v>
+        <x:v>46264.333333333336</x:v>
       </x:c>
       <x:c r="D20" s="12" t="str">
-        <x:v>千万美元</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E20" s="12" t="str">
-        <x:v>种子轮</x:v>
+        <x:v>B 轮</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="G20" s="14" t="n">
-        <x:v>7200</x:v>
-      </x:c>
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G20" s="14"/>
       <x:c r="H20" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I20" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/568250.shtml</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J20" s="15" t="n">
         <x:v>46272.77361111111</x:v>
@@ -1081,135 +1083,133 @@
         <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L20" s="12" t="str">
-        <x:v>瞬适科技（InstAdapt）聚焦具身智能与物理 AI 数据基础设施，提供真实物理世界数据采集、标注、训练与评测相关能力。公司面向机器人、自动驾驶和空间智能等场景，帮助模型更快适应动态环境。</x:v>
+        <x:v>沐创集成电路专注智能网卡、DPU 和高速互联芯片研发，面向数据中心、云计算和智算基础设施提供网络与数据处理芯片。公司产品服务高吞吐、低延迟的数据传输和计算卸载场景。</x:v>
       </x:c>
       <x:c r="M20" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.mucse.com/</x:v>
       </x:c>
       <x:c r="N20" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官网联系页：https://www.mucse.com/contact.html</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="12" t="str">
-        <x:v>灵初智能</x:v>
+        <x:v>研微半导体</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
-        <x:v>具身智能 / 机器人</x:v>
+        <x:v>半导体设备 / 薄膜沉积</x:v>
       </x:c>
       <x:c r="C21" s="13" t="n">
-        <x:v>46261.333333333336</x:v>
+        <x:v>46264.333333333336</x:v>
       </x:c>
       <x:c r="D21" s="12" t="str">
-        <x:v>过亿美元</x:v>
+        <x:v>近15亿元人民币</x:v>
       </x:c>
       <x:c r="E21" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>B 轮</x:v>
       </x:c>
       <x:c r="F21" s="12" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="G21" s="14" t="n">
-        <x:v>72000</x:v>
-      </x:c>
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G21" s="14"/>
       <x:c r="H21" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I21" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%81%B5%E5%88%9D%E6%99%BA%E8%83%BD%20%E8%BF%87%E4%BA%BF%E7%BE%8E%E5%85%83%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J21" s="15" t="n">
-        <x:v>46272.748611111114</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K21" s="12" t="str">
-        <x:v>媒体核验；官网待交叉确认</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L21" s="12" t="str">
-        <x:v>灵初智能专注具身智能与机器人基础模型，研发面向真实物理世界操作的感知、决策和控制系统。公司目标是通过大模型、仿真训练和机器人本体能力结合，提升通用机器人在工业、服务和家庭场景中的可用性。</x:v>
+        <x:v>研微半导体聚焦半导体薄膜沉积设备和关键制程装备研发，服务集成电路、先进封装和泛半导体制造。公司围绕国产半导体设备替代、工艺适配和产线交付推进产业化。</x:v>
       </x:c>
       <x:c r="M21" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.psrsemi.com/</x:v>
       </x:c>
       <x:c r="N21" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官网联系页：https://www.psrsemi.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="12" t="str">
-        <x:v>晰见科技</x:v>
+        <x:v>迈步机器人</x:v>
       </x:c>
       <x:c r="B22" s="12" t="str">
-        <x:v>类脑视觉芯片 / 物理 AI</x:v>
+        <x:v>康复机器人 / 外骨骼</x:v>
       </x:c>
       <x:c r="C22" s="13" t="n">
-        <x:v>46261.333333333336</x:v>
+        <x:v>46264.333333333336</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
-        <x:v>近5亿元人民币</x:v>
+        <x:v>近亿元人民币</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>连续3轮融资</x:v>
+        <x:v>战略融资</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G22" s="14"/>
       <x:c r="H22" s="12" t="str">
-        <x:v>新浪财经 / 投资界</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I22" s="16" t="str">
-        <x:v>https://finance.sina.com.cn/jjxw/2026-08-27/doc-iniptnuz5849968.shtml</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J22" s="15" t="n">
         <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K22" s="12" t="str">
-        <x:v>媒体与公开官网信息交叉核验</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L22" s="12" t="str">
-        <x:v>晰见科技围绕类脑视觉芯片和物理 AI 计算架构开展研发，产品面向低功耗视觉感知、机器人和边缘智能场景。公司试图通过传感、计算和算法协同提升机器在真实环境中的视觉处理效率。</x:v>
+        <x:v>迈步机器人是一家康复机器人和外骨骼设备企业，产品覆盖下肢康复训练、步态训练和智能辅助行走等方向。公司面向医院、康复中心和家庭康复场景，结合机器人控制、传感和康复医学提升训练效率。</x:v>
       </x:c>
       <x:c r="M22" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.milebot.com/</x:v>
       </x:c>
       <x:c r="N22" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官网联系页：https://www.milebot.com/contact.html</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="12" t="str">
-        <x:v>艾联纳医药</x:v>
+        <x:v>屹艮科技</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
-        <x:v>创新药 / 小分子药物</x:v>
+        <x:v>AI for Science / 电池设计自动化</x:v>
       </x:c>
       <x:c r="C23" s="13" t="n">
-        <x:v>46261.333333333336</x:v>
+        <x:v>46264.333333333336</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
-        <x:v>超1亿元人民币</x:v>
+        <x:v>亿元级人民币</x:v>
       </x:c>
       <x:c r="E23" s="12" t="str">
-        <x:v>Seed+ 轮</x:v>
+        <x:v>战略融资</x:v>
       </x:c>
       <x:c r="F23" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G23" s="14"/>
       <x:c r="H23" s="12" t="str">
-        <x:v>大河财立方</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I23" s="16" t="str">
-        <x:v>https://m.sohu.com/a/1068278269_120109837?scm=10001.325_13-325_13.0.0-0-0-0-0.5_1334</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J23" s="15" t="n">
         <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K23" s="12" t="str">
-        <x:v>媒体交叉核验；官网待确认</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L23" s="12" t="str">
-        <x:v>艾联纳医药是一家创新药研发企业，围绕小分子药物发现和疾病靶点验证推进早期管线。公司重点建设药物设计、转化研究和临床前开发能力，服务肿瘤、免疫或其他高未满足需求疾病方向。</x:v>
+        <x:v>屹艮科技面向电池材料研发和电池设计自动化建设 AI for Science 平台，支持材料筛选、配方设计和性能预测。公司将机器学习、实验数据和多尺度仿真结合，服务新能源电池研发效率提升。</x:v>
       </x:c>
       <x:c r="M23" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1220,16 +1220,16 @@
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="12" t="str">
-        <x:v>蜂巢互联</x:v>
+        <x:v>中数睿智</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
-        <x:v>工业软件 / 物理 AI 仿真</x:v>
+        <x:v>大模型 / 企业 AI Agent</x:v>
       </x:c>
       <x:c r="C24" s="13" t="n">
-        <x:v>46260.333333333336</x:v>
+        <x:v>46264.333333333336</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>12亿元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E24" s="12" t="str">
         <x:v>战略融资</x:v>
@@ -1237,98 +1237,98 @@
       <x:c r="F24" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G24" s="14" t="n">
-        <x:v>120000</x:v>
-      </x:c>
+      <x:c r="G24" s="14"/>
       <x:c r="H24" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I24" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E8%9C%82%E5%B7%A2%E4%BA%92%E8%81%94%2012%E4%BA%BF%E5%85%83%20%E8%9E%8D%E8%B5%84%20%E7%89%A9%E7%90%86AI%E4%BB%BF%E7%9C%9F%E5%BC%95%E6%93%8E&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J24" s="15" t="n">
-        <x:v>46272.748611111114</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K24" s="12" t="str">
         <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L24" s="12" t="str">
-        <x:v>蜂巢互联提供工业软件、数字孪生和物理 AI 仿真能力，面向制造业复杂设备和产线构建虚实融合平台。公司通过仿真引擎、工业互联网和数据模型，支持研发验证、生产优化和智能运维场景。</x:v>
+        <x:v>中数睿智聚焦企业级大模型和 AI Agent 应用，推出语思等面向行业知识、办公协同和智能决策的产品体系。公司服务政府、央国企和大型组织的数字化与智能化升级场景。</x:v>
       </x:c>
       <x:c r="M24" s="12" t="str">
-        <x:v>https://www.vbullet.com/</x:v>
+        <x:v>https://www.zhongshuruizhi.com/</x:v>
       </x:c>
       <x:c r="N24" s="12" t="str">
-        <x:v>官网联系页：https://www.vbullet.com/</x:v>
+        <x:v>官网联系页：https://www.zhongshuruizhi.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="12" t="str">
-        <x:v>原力引擎</x:v>
+        <x:v>星邑空间</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
-        <x:v>AI for Engineering / 生成式仿真</x:v>
+        <x:v>商业航天 / 卫星测运控</x:v>
       </x:c>
       <x:c r="C25" s="13" t="n">
-        <x:v>46260.333333333336</x:v>
+        <x:v>46264.333333333336</x:v>
       </x:c>
       <x:c r="D25" s="12" t="str">
-        <x:v>近5000万元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E25" s="12" t="str">
-        <x:v>天使+轮</x:v>
+        <x:v>A 轮增资扩股</x:v>
       </x:c>
       <x:c r="F25" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G25" s="14"/>
       <x:c r="H25" s="12" t="str">
-        <x:v>新浪财经</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I25" s="16" t="str">
-        <x:v>https://finance.sina.cn/2026-08-26/detail-inipqwax2358348.d.html</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J25" s="15" t="n">
         <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K25" s="12" t="str">
-        <x:v>媒体核验；官网待交叉确认</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L25" s="12" t="str">
-        <x:v>原力引擎聚焦 AI for Engineering 和生成式仿真，面向工程研发提供仿真建模、设计探索和智能优化工具。公司希望用大模型与数值仿真结合，提升工业研发、装备设计和复杂系统工程效率。</x:v>
+        <x:v>星邑空间从事商业航天测运控、卫星数据服务和空间信息基础设施建设，面向卫星运营、遥感应用和低轨星座服务提供能力。公司围绕地面站网络、测控调度和空间数据应用推进商业化。</x:v>
       </x:c>
       <x:c r="M25" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.xingyispace.com/</x:v>
       </x:c>
       <x:c r="N25" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官网联系页：https://www.xingyispace.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="12" t="str">
-        <x:v>赛科动力</x:v>
+        <x:v>瞬适科技</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
-        <x:v>固态电池</x:v>
+        <x:v>具身智能 / 物理 AI 数据基础设施</x:v>
       </x:c>
       <x:c r="C26" s="13" t="n">
-        <x:v>46260.333333333336</x:v>
+        <x:v>46262.333333333336</x:v>
       </x:c>
       <x:c r="D26" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>千万美元</x:v>
       </x:c>
       <x:c r="E26" s="12" t="str">
-        <x:v>股权融资</x:v>
+        <x:v>种子轮</x:v>
       </x:c>
       <x:c r="F26" s="12" t="str">
-        <x:v>CNY</x:v>
-      </x:c>
-      <x:c r="G26" s="14"/>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G26" s="14" t="n">
+        <x:v>7200</x:v>
+      </x:c>
       <x:c r="H26" s="12" t="str">
-        <x:v>园区世界投融资周报</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I26" s="16" t="str">
-        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
+        <x:v>https://news.pedaily.cn/202608/568250.shtml</x:v>
       </x:c>
       <x:c r="J26" s="15" t="n">
         <x:v>46272.77361111111</x:v>
@@ -1337,7 +1337,7 @@
         <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L26" s="12" t="str">
-        <x:v>赛科动力专注固态电池技术研发与产业化，围绕高安全、高能量密度电池材料、工艺和电芯产品推进量产。公司面向新能源汽车、低空飞行器、储能和消费电子等应用场景。</x:v>
+        <x:v>瞬适科技（InstAdapt）聚焦具身智能与物理 AI 数据基础设施，提供真实物理世界数据采集、标注、训练与评测相关能力。公司面向机器人、自动驾驶和空间智能等场景，帮助模型更快适应动态环境。</x:v>
       </x:c>
       <x:c r="M26" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1348,38 +1348,40 @@
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="12" t="str">
-        <x:v>简智机器人</x:v>
+        <x:v>灵初智能</x:v>
       </x:c>
       <x:c r="B27" s="12" t="str">
-        <x:v>具身智能 / 数据基础设施</x:v>
+        <x:v>具身智能 / 机器人</x:v>
       </x:c>
       <x:c r="C27" s="13" t="n">
-        <x:v>46260.333333333336</x:v>
+        <x:v>46261.333333333336</x:v>
       </x:c>
       <x:c r="D27" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>过亿美元</x:v>
       </x:c>
       <x:c r="E27" s="12" t="str">
         <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F27" s="12" t="str">
-        <x:v>CNY</x:v>
-      </x:c>
-      <x:c r="G27" s="14"/>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G27" s="14" t="n">
+        <x:v>72000</x:v>
+      </x:c>
       <x:c r="H27" s="12" t="str">
-        <x:v>园区世界投融资周报</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I27" s="16" t="str">
-        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
+        <x:v>https://news.google.com/search?q=%E7%81%B5%E5%88%9D%E6%99%BA%E8%83%BD%20%E8%BF%87%E4%BA%BF%E7%BE%8E%E5%85%83%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J27" s="15" t="n">
-        <x:v>46272.77361111111</x:v>
+        <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K27" s="12" t="str">
         <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L27" s="12" t="str">
-        <x:v>简智机器人围绕具身智能数据基础设施和机器人数据闭环构建平台能力，支持机器人模型训练、评测与部署。公司面向通用机器人、工业机器人和智能体开发场景，强调高质量数据和模型迭代效率。</x:v>
+        <x:v>灵初智能专注具身智能与机器人基础模型，研发面向真实物理世界操作的感知、决策和控制系统。公司目标是通过大模型、仿真训练和机器人本体能力结合，提升通用机器人在工业、服务和家庭场景中的可用性。</x:v>
       </x:c>
       <x:c r="M27" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1390,82 +1392,80 @@
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="12" t="str">
-        <x:v>小鹏机器人</x:v>
+        <x:v>晰见科技</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
-        <x:v>人形机器人 / 具身智能</x:v>
+        <x:v>类脑视觉芯片 / 物理 AI</x:v>
       </x:c>
       <x:c r="C28" s="13" t="n">
-        <x:v>46258.333333333336</x:v>
+        <x:v>46261.333333333336</x:v>
       </x:c>
       <x:c r="D28" s="12" t="str">
-        <x:v>超9亿美元</x:v>
+        <x:v>近5亿元人民币</x:v>
       </x:c>
       <x:c r="E28" s="12" t="str">
-        <x:v>首轮融资</x:v>
+        <x:v>连续3轮融资</x:v>
       </x:c>
       <x:c r="F28" s="12" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="G28" s="14" t="n">
-        <x:v>648000</x:v>
-      </x:c>
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G28" s="14"/>
       <x:c r="H28" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>新浪财经 / 投资界</x:v>
       </x:c>
       <x:c r="I28" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%B0%8F%E9%B9%8F%E6%9C%BA%E5%99%A8%E4%BA%BA%20%E8%B6%859%E4%BA%BF%E7%BE%8E%E5%85%83%20%E9%A6%96%E8%BD%AE%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://finance.sina.com.cn/jjxw/2026-08-27/doc-iniptnuz5849968.shtml</x:v>
       </x:c>
       <x:c r="J28" s="15" t="n">
-        <x:v>46272.748611111114</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K28" s="12" t="str">
-        <x:v>媒体交叉核验</x:v>
+        <x:v>媒体与公开官网信息交叉核验</x:v>
       </x:c>
       <x:c r="L28" s="12" t="str">
-        <x:v>小鹏机器人是小鹏体系内面向人形机器人和具身智能方向的业务，公开展示过 IRON 等机器人产品。其研发围绕机器人本体、运动控制、环境感知和智能交互展开，目标是将智能汽车相关技术能力延伸到机器人场景。</x:v>
+        <x:v>晰见科技围绕类脑视觉芯片和物理 AI 计算架构开展研发，产品面向低功耗视觉感知、机器人和边缘智能场景。公司试图通过传感、计算和算法协同提升机器在真实环境中的视觉处理效率。</x:v>
       </x:c>
       <x:c r="M28" s="12" t="str">
-        <x:v>https://www.xpeng.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N28" s="12" t="str">
-        <x:v>官网联系页：https://www.xpeng.com/contact</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="12" t="str">
-        <x:v>枢途科技</x:v>
+        <x:v>艾联纳医药</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
-        <x:v>AGI Infra / AI 数据基础设施</x:v>
+        <x:v>创新药 / 小分子药物</x:v>
       </x:c>
       <x:c r="C29" s="13" t="n">
-        <x:v>46258.333333333336</x:v>
+        <x:v>46261.333333333336</x:v>
       </x:c>
       <x:c r="D29" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>超1亿元人民币</x:v>
       </x:c>
       <x:c r="E29" s="12" t="str">
-        <x:v>连续两轮融资</x:v>
+        <x:v>Seed+ 轮</x:v>
       </x:c>
       <x:c r="F29" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G29" s="14"/>
       <x:c r="H29" s="12" t="str">
-        <x:v>36氪</x:v>
+        <x:v>大河财立方</x:v>
       </x:c>
       <x:c r="I29" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%9E%A2%E9%80%94%E7%A7%91%E6%8A%80%20%E8%BF%9E%E7%BB%AD%E5%AE%8C%E6%88%90%E4%B8%A4%E8%BD%AE%E8%9E%8D%E8%B5%84%202026&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://m.sohu.com/a/1068278269_120109837?scm=10001.325_13-325_13.0.0-0-0-0-0.5_1334</x:v>
       </x:c>
       <x:c r="J29" s="15" t="n">
-        <x:v>46272.748611111114</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K29" s="12" t="str">
-        <x:v>媒体核验；官网待交叉确认</x:v>
+        <x:v>媒体交叉核验；官网待确认</x:v>
       </x:c>
       <x:c r="L29" s="12" t="str">
-        <x:v>枢途科技聚焦 AGI Infra 与 AI 数据基础设施，面向大模型训练、智能体开发和企业 AI 应用提供底层数据与工程平台。公司强调数据流、知识组织和模型应用之间的连接能力，帮助团队更高效地构建可落地的智能系统。</x:v>
+        <x:v>艾联纳医药是一家创新药研发企业，围绕小分子药物发现和疾病靶点验证推进早期管线。公司重点建设药物设计、转化研究和临床前开发能力，服务肿瘤、免疫或其他高未满足需求疾病方向。</x:v>
       </x:c>
       <x:c r="M29" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1476,144 +1476,144 @@
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="12" t="str">
-        <x:v>中科第五纪</x:v>
+        <x:v>蜂巢互联</x:v>
       </x:c>
       <x:c r="B30" s="12" t="str">
-        <x:v>具身智能 / 具身大脑</x:v>
+        <x:v>工业软件 / 物理 AI 仿真</x:v>
       </x:c>
       <x:c r="C30" s="13" t="n">
-        <x:v>46254.333333333336</x:v>
+        <x:v>46260.333333333336</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>超10亿元人民币</x:v>
+        <x:v>12亿元人民币</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
-        <x:v>A1、A2 轮</x:v>
+        <x:v>战略融资</x:v>
       </x:c>
       <x:c r="F30" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G30" s="14"/>
+      <x:c r="G30" s="14" t="n">
+        <x:v>120000</x:v>
+      </x:c>
       <x:c r="H30" s="12" t="str">
-        <x:v>科创板日报 / 东方财富</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I30" s="16" t="str">
-        <x:v>https://finance.eastmoney.com/a/202608203847689590.html</x:v>
+        <x:v>https://news.google.com/search?q=%E8%9C%82%E5%B7%A2%E4%BA%92%E8%81%94%2012%E4%BA%BF%E5%85%83%20%E8%9E%8D%E8%B5%84%20%E7%89%A9%E7%90%86AI%E4%BB%BF%E7%9C%9F%E5%BC%95%E6%93%8E&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J30" s="15" t="n">
-        <x:v>46272.77361111111</x:v>
+        <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K30" s="12" t="str">
-        <x:v>媒体核验；官网待交叉确认</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L30" s="12" t="str">
-        <x:v>中科第五纪专注具身智能和具身大脑技术，围绕机器人感知、决策、动作生成和世界模型构建基础能力。公司面向通用机器人、工业智能和真实世界交互场景推进产品化。</x:v>
+        <x:v>蜂巢互联提供工业软件、数字孪生和物理 AI 仿真能力，面向制造业复杂设备和产线构建虚实融合平台。公司通过仿真引擎、工业互联网和数据模型，支持研发验证、生产优化和智能运维场景。</x:v>
       </x:c>
       <x:c r="M30" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.vbullet.com/</x:v>
       </x:c>
       <x:c r="N30" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官网联系页：https://www.vbullet.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="12" t="str">
-        <x:v>嘉腾机器人</x:v>
+        <x:v>原力引擎</x:v>
       </x:c>
       <x:c r="B31" s="12" t="str">
-        <x:v>工业具身智能 / AGV / AMR</x:v>
+        <x:v>AI for Engineering / 生成式仿真</x:v>
       </x:c>
       <x:c r="C31" s="13" t="n">
-        <x:v>46252.333333333336</x:v>
+        <x:v>46260.333333333336</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
-        <x:v>数千万元人民币</x:v>
+        <x:v>近5000万元人民币</x:v>
       </x:c>
       <x:c r="E31" s="12" t="str">
-        <x:v>战略融资</x:v>
+        <x:v>天使+轮</x:v>
       </x:c>
       <x:c r="F31" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G31" s="14"/>
       <x:c r="H31" s="12" t="str">
-        <x:v>21世纪经济报道</x:v>
+        <x:v>新浪财经</x:v>
       </x:c>
       <x:c r="I31" s="16" t="str">
-        <x:v>https://m.21jingji.com/article/20260818/herald/09ad8c401fbb711d0cd6717d4988613c.html</x:v>
+        <x:v>https://finance.sina.cn/2026-08-26/detail-inipqwax2358348.d.html</x:v>
       </x:c>
       <x:c r="J31" s="15" t="n">
-        <x:v>46253.82167824074</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K31" s="12" t="str">
-        <x:v>媒体交叉核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L31" s="12" t="str">
-        <x:v>嘉腾机器人专注工业自动化解决方案与机器人研发制造，重点布局 AGV、AMR 及具身智能移动底盘等产品。公司面向制造、仓储、物流与工业搬运场景，强调规模化交付和全球化应用能力。</x:v>
+        <x:v>原力引擎聚焦 AI for Engineering 和生成式仿真，面向工程研发提供仿真建模、设计探索和智能优化工具。公司希望用大模型与数值仿真结合，提升工业研发、装备设计和复杂系统工程效率。</x:v>
       </x:c>
       <x:c r="M31" s="12" t="str">
-        <x:v>https://www.jtrobots.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N31" s="12" t="str">
-        <x:v>总机电话：400-830-1028；商务邮箱：marketing@jtrobots.com；官网联系页：https://www.jtrobots.com/address</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="12" t="str">
-        <x:v>灵锶智能</x:v>
+        <x:v>赛科动力</x:v>
       </x:c>
       <x:c r="B32" s="12" t="str">
-        <x:v>四足机器人 / 人形机器人</x:v>
+        <x:v>固态电池</x:v>
       </x:c>
       <x:c r="C32" s="13" t="n">
-        <x:v>46252.333333333336</x:v>
+        <x:v>46260.333333333336</x:v>
       </x:c>
       <x:c r="D32" s="12" t="str">
-        <x:v>7000万元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E32" s="12" t="str">
-        <x:v>战略融资</x:v>
+        <x:v>股权融资</x:v>
       </x:c>
       <x:c r="F32" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G32" s="14" t="n">
-        <x:v>7000</x:v>
-      </x:c>
+      <x:c r="G32" s="14"/>
       <x:c r="H32" s="12" t="str">
-        <x:v>新浪科技</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I32" s="16" t="str">
-        <x:v>https://finance.sina.com.cn/tech/roll/2026-08-18/doc-inintpin8618761.shtml</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J32" s="15" t="n">
-        <x:v>46253.82167824074</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K32" s="12" t="str">
-        <x:v>媒体交叉核验</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L32" s="12" t="str">
-        <x:v>灵锶智能聚焦四足机器人与人形 AI 机器人研发，产品面向电力巡检、应急救援、工厂巡检等复杂工业场景。公司强调重载、长续航和复杂地形适应能力，并在广东机器人产业链中持续推进产品化。</x:v>
+        <x:v>赛科动力专注固态电池技术研发与产业化，围绕高安全、高能量密度电池材料、工艺和电芯产品推进量产。公司面向新能源汽车、低空飞行器、储能和消费电子等应用场景。</x:v>
       </x:c>
       <x:c r="M32" s="12" t="str">
-        <x:v>https://www.gdlinxai.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N32" s="12" t="str">
-        <x:v>电话：17710125211；邮箱：info@linxai-tech.com；官网联系页：https://www.gdlinxai.com/h-col-109.html</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="12" t="str">
-        <x:v>安澜德健</x:v>
+        <x:v>简智机器人</x:v>
       </x:c>
       <x:c r="B33" s="12" t="str">
-        <x:v>医疗器械 / 心室辅助装置</x:v>
+        <x:v>具身智能 / 数据基础设施</x:v>
       </x:c>
       <x:c r="C33" s="13" t="n">
-        <x:v>46252.333333333336</x:v>
+        <x:v>46260.333333333336</x:v>
       </x:c>
       <x:c r="D33" s="12" t="str">
-        <x:v>近亿元人民币</x:v>
+        <x:v>未披露</x:v>
       </x:c>
       <x:c r="E33" s="12" t="str">
         <x:v>A 轮</x:v>
@@ -1623,298 +1623,298 @@
       </x:c>
       <x:c r="G33" s="14"/>
       <x:c r="H33" s="12" t="str">
-        <x:v>启明创投</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I33" s="16" t="str">
-        <x:v>https://www.qimingvc.com/cn/news/%E5%90%AF%E6%98%8E%E6%98%9F-%E5%AE%89%E6%BE%9C%E5%BE%B7%E5%81%A5%E5%AE%8C%E6%88%90%E8%BF%91%E4%BA%BF%E5%85%83a%E8%BD%AE%E8%9E%8D%E8%B5%84%EF%BC%8C%E5%90%AF%E6%98%8E%E5%88%9B%E6%8A%95%E7%8B%AC%E5%AE%B6%E6%8A%95%E8%B5%84</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J33" s="15" t="n">
-        <x:v>46253.82167824074</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K33" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L33" s="12" t="str">
-        <x:v>安澜德健（Enginprime Medical）专注经皮心室辅助装置（pVAD）研发，核心产品为 OpusOne™。公司围绕更小尺寸、更高流量的心室辅助系统推进中国注册临床试验与海外早期临床申报。</x:v>
+        <x:v>简智机器人围绕具身智能数据基础设施和机器人数据闭环构建平台能力，支持机器人模型训练、评测与部署。公司面向通用机器人、工业机器人和智能体开发场景，强调高质量数据和模型迭代效率。</x:v>
       </x:c>
       <x:c r="M33" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N33" s="12" t="str">
-        <x:v>媒体邮箱：media@enginprime.com；投资者联系：info@voyagerscap.com</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="12" t="str">
-        <x:v>亿兰科</x:v>
+        <x:v>小鹏机器人</x:v>
       </x:c>
       <x:c r="B34" s="12" t="str">
-        <x:v>高端分析仪器 / 质谱仪</x:v>
+        <x:v>人形机器人 / 具身智能</x:v>
       </x:c>
       <x:c r="C34" s="13" t="n">
-        <x:v>46245.333333333336</x:v>
+        <x:v>46258.333333333336</x:v>
       </x:c>
       <x:c r="D34" s="12" t="str">
-        <x:v>数千万元人民币</x:v>
+        <x:v>超9亿美元</x:v>
       </x:c>
       <x:c r="E34" s="12" t="str">
-        <x:v>Pre-A 轮</x:v>
+        <x:v>首轮融资</x:v>
       </x:c>
       <x:c r="F34" s="12" t="str">
-        <x:v>CNY</x:v>
-      </x:c>
-      <x:c r="G34" s="14"/>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G34" s="14" t="n">
+        <x:v>648000</x:v>
+      </x:c>
       <x:c r="H34" s="12" t="str">
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I34" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/567473.shtml</x:v>
+        <x:v>https://news.google.com/search?q=%E5%B0%8F%E9%B9%8F%E6%9C%BA%E5%99%A8%E4%BA%BA%20%E8%B6%859%E4%BA%BF%E7%BE%8E%E5%85%83%20%E9%A6%96%E8%BD%AE%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J34" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K34" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体交叉核验</x:v>
       </x:c>
       <x:c r="L34" s="12" t="str">
-        <x:v>亿兰科专注工商业模块化光储系统和电力电子设备，围绕 PCS、混合逆变器、光储一体机与微电网管理系统开展研发和交付。公司产品服务工商业储能、分布式光伏和海外终端市场。</x:v>
+        <x:v>小鹏机器人是小鹏体系内面向人形机器人和具身智能方向的业务，公开展示过 IRON 等机器人产品。其研发围绕机器人本体、运动控制、环境感知和智能交互展开，目标是将智能汽车相关技术能力延伸到机器人场景。</x:v>
       </x:c>
       <x:c r="M34" s="12" t="str">
-        <x:v>https://www.elecod.cn/</x:v>
+        <x:v>https://www.xpeng.com/</x:v>
       </x:c>
       <x:c r="N34" s="12" t="str">
-        <x:v>电话：0755-23050802；商务邮箱：marketing@elecod.com；人力邮箱：hr@elecod.com；官网联系页：https://www.elecod.cn/aboutus.html。</x:v>
+        <x:v>官网联系页：https://www.xpeng.com/contact</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="12" t="str">
-        <x:v>诺因智能</x:v>
+        <x:v>枢途科技</x:v>
       </x:c>
       <x:c r="B35" s="12" t="str">
-        <x:v>具身智能 / 消费级机器人</x:v>
+        <x:v>AGI Infra / AI 数据基础设施</x:v>
       </x:c>
       <x:c r="C35" s="13" t="n">
-        <x:v>46244.333333333336</x:v>
+        <x:v>46258.333333333336</x:v>
       </x:c>
       <x:c r="D35" s="12" t="str">
-        <x:v>5 亿元人民币</x:v>
+        <x:v>未披露</x:v>
       </x:c>
       <x:c r="E35" s="12" t="str">
-        <x:v>天使++轮</x:v>
+        <x:v>连续两轮融资</x:v>
       </x:c>
       <x:c r="F35" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G35" s="14" t="n">
-        <x:v>50000</x:v>
-      </x:c>
+      <x:c r="G35" s="14"/>
       <x:c r="H35" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>36氪</x:v>
       </x:c>
       <x:c r="I35" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/567457.shtml</x:v>
+        <x:v>https://news.google.com/search?q=%E6%9E%A2%E9%80%94%E7%A7%91%E6%8A%80%20%E8%BF%9E%E7%BB%AD%E5%AE%8C%E6%88%90%E4%B8%A4%E8%BD%AE%E8%9E%8D%E8%B5%84%202026&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J35" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K35" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L35" s="12" t="str">
-        <x:v>诺因智能聚焦家庭场景具身智能，围绕折叠双臂机器人及相关感知、执行和交互系统推进产品研发。公司目标是让机器人进入真实家庭环境，承担陪伴互动、整理和基础协作等任务。</x:v>
+        <x:v>枢途科技聚焦触觉技术和具身智能数据基础设施，研发 SynaTac 等触觉技术与产品，并提供人类行为数据采集和交付能力。公司面向机器人接触智能、生命科学和具身智能训练场景，建设从数据生产到机器人应用的技术链路。</x:v>
       </x:c>
       <x:c r="M35" s="12" t="str">
-        <x:v>https://knowinai.com/</x:v>
+        <x:v>https://www.synapath.com/</x:v>
       </x:c>
       <x:c r="N35" s="12" t="str">
-        <x:v>招聘邮箱：HR@knowin.ai；联系电话：17610340223；媒介合作：media@knowin.ai；官方联系页：https://knowinai.com/。</x:v>
+        <x:v>官网已核验；未检索到公开商务邮箱或电话，可通过官网联系入口咨询。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="12" t="str">
-        <x:v>星环聚能</x:v>
+        <x:v>中科第五纪</x:v>
       </x:c>
       <x:c r="B36" s="12" t="str">
-        <x:v>可控聚变 / 清洁能源</x:v>
+        <x:v>具身智能 / 具身大脑</x:v>
       </x:c>
       <x:c r="C36" s="13" t="n">
-        <x:v>46244.333333333336</x:v>
+        <x:v>46254.333333333336</x:v>
       </x:c>
       <x:c r="D36" s="12" t="str">
-        <x:v>8.8 亿元人民币</x:v>
+        <x:v>超10亿元人民币</x:v>
       </x:c>
       <x:c r="E36" s="12" t="str">
-        <x:v>A++ 轮</x:v>
+        <x:v>A1、A2 轮</x:v>
       </x:c>
       <x:c r="F36" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G36" s="14" t="n">
-        <x:v>88000</x:v>
-      </x:c>
+      <x:c r="G36" s="14"/>
       <x:c r="H36" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>科创板日报 / 东方财富</x:v>
       </x:c>
       <x:c r="I36" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/567446.shtml</x:v>
+        <x:v>https://finance.eastmoney.com/a/202608203847689590.html</x:v>
       </x:c>
       <x:c r="J36" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K36" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L36" s="12" t="str">
-        <x:v>星环聚能专注可控核聚变相关技术和工程化系统，推动聚变能装备研发及商业化路径。公司面向清洁能源、长期稳定供能和能源转型场景，持续扩展实验和产业化能力。</x:v>
+        <x:v>中科第五纪专注具身智能和具身大脑技术，围绕机器人感知、决策、动作生成和世界模型构建基础能力。公司面向通用机器人、工业智能和真实世界交互场景推进产品化。</x:v>
       </x:c>
       <x:c r="M36" s="12" t="str">
-        <x:v>https://startorus.cn/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N36" s="12" t="str">
-        <x:v>电话：029-86041002；邮箱：business@startorus.cn；公司地址：上海市嘉定区澄浏公路52号39幢2楼JT109869室；官网联系页：https://startorus.cn/。</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="12" t="str">
-        <x:v>奇算光启</x:v>
+        <x:v>嘉腾机器人</x:v>
       </x:c>
       <x:c r="B37" s="12" t="str">
-        <x:v>AI 光计算芯片</x:v>
+        <x:v>工业具身智能 / AGV / AMR</x:v>
       </x:c>
       <x:c r="C37" s="13" t="n">
-        <x:v>46244.333333333336</x:v>
+        <x:v>46252.333333333336</x:v>
       </x:c>
       <x:c r="D37" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E37" s="12" t="str">
-        <x:v>天使轮及天使+轮</x:v>
+        <x:v>战略融资</x:v>
       </x:c>
       <x:c r="F37" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G37" s="14"/>
       <x:c r="H37" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>21世纪经济报道</x:v>
       </x:c>
       <x:c r="I37" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/567453.shtml</x:v>
+        <x:v>https://m.21jingji.com/article/20260818/herald/09ad8c401fbb711d0cd6717d4988613c.html</x:v>
       </x:c>
       <x:c r="J37" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46253.82167824074</x:v>
       </x:c>
       <x:c r="K37" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体交叉核验</x:v>
       </x:c>
       <x:c r="L37" s="12" t="str">
-        <x:v>奇算光启专注 AI 光计算芯片和光计算系统研发，试图用全光计算与集成光子技术突破传统电子芯片能效瓶颈。公司面向大模型和高性能计算底座，强调算力密度、功耗和系统扩展能力。</x:v>
+        <x:v>嘉腾机器人专注工业自动化解决方案与机器人研发制造，重点布局 AGV、AMR 及具身智能移动底盘等产品。公司面向制造、仓储、物流与工业搬运场景，强调规模化交付和全球化应用能力。</x:v>
       </x:c>
       <x:c r="M37" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.jtrobots.com/</x:v>
       </x:c>
       <x:c r="N37" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>总机电话：400-830-1028；商务邮箱：marketing@jtrobots.com；官网联系页：https://www.jtrobots.com/address</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="12" t="str">
-        <x:v>深度细胞</x:v>
+        <x:v>灵锶智能</x:v>
       </x:c>
       <x:c r="B38" s="12" t="str">
-        <x:v>AI 医疗 / 单细胞分析</x:v>
+        <x:v>四足机器人 / 人形机器人</x:v>
       </x:c>
       <x:c r="C38" s="13" t="n">
-        <x:v>46244.333333333336</x:v>
+        <x:v>46252.333333333336</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
-        <x:v>近亿元人民币</x:v>
+        <x:v>7000万元人民币</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
-        <x:v>种子轮</x:v>
+        <x:v>战略融资</x:v>
       </x:c>
       <x:c r="F38" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G38" s="14"/>
+      <x:c r="G38" s="14" t="n">
+        <x:v>7000</x:v>
+      </x:c>
       <x:c r="H38" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>新浪科技</x:v>
       </x:c>
       <x:c r="I38" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/567451.shtml</x:v>
+        <x:v>https://finance.sina.com.cn/tech/roll/2026-08-18/doc-inintpin8618761.shtml</x:v>
       </x:c>
       <x:c r="J38" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46253.82167824074</x:v>
       </x:c>
       <x:c r="K38" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体交叉核验</x:v>
       </x:c>
       <x:c r="L38" s="12" t="str">
-        <x:v>深度细胞聚焦 AI 制药与虚拟细胞建模，围绕单细胞分析、疾病机理和药物研发加速构建算法平台。公司目标是把细胞级计算能力用于新药发现和生物医学研究。</x:v>
+        <x:v>灵锶智能聚焦四足机器人与人形 AI 机器人研发，产品面向电力巡检、应急救援、工厂巡检等复杂工业场景。公司强调重载、长续航和复杂地形适应能力，并在广东机器人产业链中持续推进产品化。</x:v>
       </x:c>
       <x:c r="M38" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.gdlinxai.com/</x:v>
       </x:c>
       <x:c r="N38" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>电话：17710125211；邮箱：info@linxai-tech.com；官网联系页：https://www.gdlinxai.com/h-col-109.html</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="12" t="str">
-        <x:v>橡木果机器人</x:v>
+        <x:v>安澜德健</x:v>
       </x:c>
       <x:c r="B39" s="12" t="str">
-        <x:v>具身智能 / 人形机器人</x:v>
+        <x:v>医疗器械 / 心室辅助装置</x:v>
       </x:c>
       <x:c r="C39" s="13" t="n">
-        <x:v>46244.333333333336</x:v>
+        <x:v>46252.333333333336</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>近亿元人民币</x:v>
       </x:c>
       <x:c r="E39" s="12" t="str">
-        <x:v>天使轮</x:v>
+        <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F39" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G39" s="14"/>
       <x:c r="H39" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>启明创投</x:v>
       </x:c>
       <x:c r="I39" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/567448.shtml</x:v>
+        <x:v>https://www.qimingvc.com/cn/news/%E5%90%AF%E6%98%8E%E6%98%9F-%E5%AE%89%E6%BE%9C%E5%BE%B7%E5%81%A5%E5%AE%8C%E6%88%90%E8%BF%91%E4%BA%BF%E5%85%83a%E8%BD%AE%E8%9E%8D%E8%B5%84%EF%BC%8C%E5%90%AF%E6%98%8E%E5%88%9B%E6%8A%95%E7%8B%AC%E5%AE%B6%E6%8A%95%E8%B5%84</x:v>
       </x:c>
       <x:c r="J39" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46253.82167824074</x:v>
       </x:c>
       <x:c r="K39" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L39" s="12" t="str">
-        <x:v>橡木果机器人专注通用具身操作，围绕触觉感知、操作基座模型和机器人执行能力构建底层技术栈。公司强调自下而上的“本能驱动”路线，目标是让机器人在真实物理环境中稳定完成操作任务。</x:v>
+        <x:v>安澜德健（Enginprime Medical）专注经皮心室辅助装置（pVAD）研发，核心产品为 OpusOne™。公司围绕更小尺寸、更高流量的心室辅助系统推进中国注册临床试验与海外早期临床申报。</x:v>
       </x:c>
       <x:c r="M39" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N39" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>媒体邮箱：media@enginprime.com；投资者联系：info@voyagerscap.com</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="12" t="str">
-        <x:v>Noiz AI</x:v>
+        <x:v>亿兰科</x:v>
       </x:c>
       <x:c r="B40" s="12" t="str">
-        <x:v>AI 语音 / 视听内容生成</x:v>
+        <x:v>高端分析仪器 / 质谱仪</x:v>
       </x:c>
       <x:c r="C40" s="13" t="n">
-        <x:v>46244.333333333336</x:v>
+        <x:v>46245.333333333336</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
         <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E40" s="12" t="str">
-        <x:v>种子轮</x:v>
+        <x:v>Pre-A 轮</x:v>
       </x:c>
       <x:c r="F40" s="12" t="str">
         <x:v>CNY</x:v>
@@ -1924,7 +1924,7 @@
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I40" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/567447.shtml</x:v>
+        <x:v>https://news.pedaily.cn/202608/567473.shtml</x:v>
       </x:c>
       <x:c r="J40" s="15" t="n">
         <x:v>46245.44097222222</x:v>
@@ -1933,420 +1933,424 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L40" s="12" t="str">
-        <x:v>Noiz AI 提供文本转语音、声音克隆和语音设计能力，面向内容创作、配音、本地化和开发者 API 场景。其产品强调情感控制、低延迟生成和多语言语音输出，服务全球化音频工作流。</x:v>
+        <x:v>亿兰科专注工商业模块化光储系统和电力电子设备，围绕 PCS、混合逆变器、光储一体机与微电网管理系统开展研发和交付。公司产品服务工商业储能、分布式光伏和海外终端市场。</x:v>
       </x:c>
       <x:c r="M40" s="12" t="str">
-        <x:v>https://noiz.ai/</x:v>
+        <x:v>https://www.elecod.cn/</x:v>
       </x:c>
       <x:c r="N40" s="12" t="str">
-        <x:v>邮箱：contact@noiz.ai；官网联系页：https://noiz.ai/。</x:v>
+        <x:v>电话：0755-23050802；商务邮箱：marketing@elecod.com；人力邮箱：hr@elecod.com；官网联系页：https://www.elecod.cn/aboutus.html。</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="12" t="str">
-        <x:v>飞声</x:v>
+        <x:v>诺因智能</x:v>
       </x:c>
       <x:c r="B41" s="12" t="str">
-        <x:v>AI 助听器 / 医疗器械</x:v>
+        <x:v>具身智能 / 消费级机器人</x:v>
       </x:c>
       <x:c r="C41" s="13" t="n">
         <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D41" s="12" t="str">
-        <x:v>数千万元人民币</x:v>
+        <x:v>5 亿元人民币</x:v>
       </x:c>
       <x:c r="E41" s="12" t="str">
-        <x:v>天使轮</x:v>
+        <x:v>天使++轮</x:v>
       </x:c>
       <x:c r="F41" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G41" s="14"/>
+      <x:c r="G41" s="14" t="n">
+        <x:v>50000</x:v>
+      </x:c>
       <x:c r="H41" s="12" t="str">
-        <x:v>36氪</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I41" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E9%A3%9E%E5%A3%B0%20AI%20%E5%8A%A9%E5%90%AC%E5%99%A8%20%E5%A4%A9%E4%BD%BF%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202608/567457.shtml</x:v>
       </x:c>
       <x:c r="J41" s="15" t="n">
         <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K41" s="12" t="str">
-        <x:v>媒体与官网交叉核验</x:v>
+        <x:v>已核验</x:v>
       </x:c>
       <x:c r="L41" s="12" t="str">
-        <x:v>飞声专注 AI 助听器与听力辅助产品，结合声学处理、语音增强和智能交互能力改善听障场景的佩戴体验。公司面向消费级与医疗级场景推进产品化，强调清晰拾音、降噪和更自然的听觉补偿。</x:v>
+        <x:v>诺因智能聚焦家庭场景具身智能，围绕折叠双臂机器人及相关感知、执行和交互系统推进产品研发。公司目标是让机器人进入真实家庭环境，承担陪伴互动、整理和基础协作等任务。</x:v>
       </x:c>
       <x:c r="M41" s="12" t="str">
-        <x:v>https://www.flysounds.cn/zh/</x:v>
+        <x:v>https://knowinai.com/</x:v>
       </x:c>
       <x:c r="N41" s="12" t="str">
-        <x:v>电话：15828225541；商务邮箱：jory@flysounds.com；地址：深圳市龙华区龙华街道清湖社区大和路356号金鼎盛科创园A栋18楼。</x:v>
+        <x:v>招聘邮箱：HR@knowin.ai；联系电话：17610340223；媒介合作：media@knowin.ai；官方联系页：https://knowinai.com/。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="12" t="str">
-        <x:v>霍德生物</x:v>
+        <x:v>星环聚能</x:v>
       </x:c>
       <x:c r="B42" s="12" t="str">
-        <x:v>细胞治疗 / 生物技术</x:v>
+        <x:v>可控聚变 / 清洁能源</x:v>
       </x:c>
       <x:c r="C42" s="13" t="n">
         <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D42" s="12" t="str">
-        <x:v>近 2 亿元人民币</x:v>
+        <x:v>8.8 亿元人民币</x:v>
       </x:c>
       <x:c r="E42" s="12" t="str">
-        <x:v>C 轮首关</x:v>
+        <x:v>A++ 轮</x:v>
       </x:c>
       <x:c r="F42" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G42" s="14"/>
+      <x:c r="G42" s="14" t="n">
+        <x:v>88000</x:v>
+      </x:c>
       <x:c r="H42" s="12" t="str">
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I42" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E9%9C%8D%E5%BE%B7%E7%94%9F%E7%89%A9%20%E8%BF%91%202%20%E4%BA%BF%E5%85%83%20C%E8%BD%AE%20%E9%A6%96%E5%85%B3&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202608/567446.shtml</x:v>
       </x:c>
       <x:c r="J42" s="15" t="n">
         <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K42" s="12" t="str">
-        <x:v>媒体与公开工商信息交叉核验</x:v>
+        <x:v>已核验</x:v>
       </x:c>
       <x:c r="L42" s="12" t="str">
-        <x:v>霍德生物工程有限公司聚焦细胞治疗和再生医学相关技术与产品，围绕研发、工艺和临床转化推进管线建设。公司在公开页面中长期披露研发动态与产品进展，面向生物医药产业化需求。</x:v>
+        <x:v>星环聚能专注可控核聚变相关技术和工程化系统，推动聚变能装备研发及商业化路径。公司面向清洁能源、长期稳定供能和能源转型场景，持续扩展实验和产业化能力。</x:v>
       </x:c>
       <x:c r="M42" s="12" t="str">
-        <x:v>https://www.hopstem.com/</x:v>
+        <x:v>https://startorus.cn/</x:v>
       </x:c>
       <x:c r="N42" s="12" t="str">
-        <x:v>电话：0571-88197776；邮箱：info@hopstem.com；官网联系页：https://www.hopstem.com/。</x:v>
+        <x:v>电话：029-86041002；邮箱：business@startorus.cn；公司地址：上海市嘉定区澄浏公路52号39幢2楼JT109869室；官网联系页：https://startorus.cn/。</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="12" t="str">
-        <x:v>可灵 AI</x:v>
+        <x:v>奇算光启</x:v>
       </x:c>
       <x:c r="B43" s="12" t="str">
-        <x:v>AI 视频大模型</x:v>
+        <x:v>AI 光计算芯片</x:v>
       </x:c>
       <x:c r="C43" s="13" t="n">
-        <x:v>46241.333333333336</x:v>
+        <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D43" s="12" t="str">
-        <x:v>近 30 亿美元</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E43" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>天使轮及天使+轮</x:v>
       </x:c>
       <x:c r="F43" s="12" t="str">
-        <x:v>USD</x:v>
+        <x:v>CNY</x:v>
       </x:c>
       <x:c r="G43" s="14"/>
       <x:c r="H43" s="12" t="str">
-        <x:v>新华网 / 经济参考报</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I43" s="16" t="str">
-        <x:v>https://www.news.cn/tech/20260807/1605ef446e5045b7ba0ee55245ce731c/c.html</x:v>
+        <x:v>https://news.pedaily.cn/202608/567453.shtml</x:v>
       </x:c>
       <x:c r="J43" s="15" t="n">
-        <x:v>46242.48541666667</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K43" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L43" s="12" t="str">
-        <x:v>可灵 AI 是面向视频生成与创作的 AI 大模型产品，支持文本、图片等输入驱动的视频内容生成和编辑。产品服务广告创意、影视内容、社交媒体和商业化营销等场景，重点提升视频生成的一致性、可控性和创作效率。</x:v>
+        <x:v>奇算光启专注 AI 光计算芯片和光计算系统研发，试图用全光计算与集成光子技术突破传统电子芯片能效瓶颈。公司面向大模型和高性能计算底座，强调算力密度、功耗和系统扩展能力。</x:v>
       </x:c>
       <x:c r="M43" s="12" t="str">
-        <x:v>https://klingai.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N43" s="12" t="str">
-        <x:v>商务联系：官网联系页</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="12" t="str">
-        <x:v>矩阵起源</x:v>
+        <x:v>深度细胞</x:v>
       </x:c>
       <x:c r="B44" s="12" t="str">
-        <x:v>企业级 AI 基础设施</x:v>
+        <x:v>AI 医疗 / 单细胞分析</x:v>
       </x:c>
       <x:c r="C44" s="13" t="n">
-        <x:v>46240.333333333336</x:v>
+        <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D44" s="12" t="str">
-        <x:v>超 1,000 万美元</x:v>
+        <x:v>近亿元人民币</x:v>
       </x:c>
       <x:c r="E44" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>种子轮</x:v>
       </x:c>
       <x:c r="F44" s="12" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="G44" s="14" t="n">
-        <x:v>7200</x:v>
-      </x:c>
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G44" s="14"/>
       <x:c r="H44" s="12" t="str">
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I44" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%9F%A9%E9%98%B5%E8%B5%B7%E6%BA%90%20%E8%B6%85%E5%8D%83%E4%B8%87%E7%BE%8E%E5%85%83%20A%E8%BD%AE%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202608/567451.shtml</x:v>
       </x:c>
       <x:c r="J44" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K44" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L44" s="12" t="str">
-        <x:v>矩阵起源专注 AI 原生数据基础设施，提供多模态数据处理、数据库与企业级 AI 数据底座产品及解决方案。其产品面向企业在结构化、非结构化和向量数据之间建立统一的数据管理与计算能力，为模型训练、知识检索和 AI 应用部署提供底层支撑。</x:v>
+        <x:v>深度细胞聚焦 AI 制药与虚拟细胞建模，围绕单细胞分析、疾病机理和药物研发加速构建算法平台。公司目标是把细胞级计算能力用于新药发现和生物医学研究。</x:v>
       </x:c>
       <x:c r="M44" s="12" t="str">
-        <x:v>https://matrixorigin.cn/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N44" s="12" t="str">
-        <x:v>商务邮箱：contact@matrixorigin.cn。</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="12" t="str">
-        <x:v>为光能源</x:v>
+        <x:v>橡木果机器人</x:v>
       </x:c>
       <x:c r="B45" s="12" t="str">
-        <x:v>电力电子 / 固态变压器</x:v>
+        <x:v>具身智能 / 人形机器人</x:v>
       </x:c>
       <x:c r="C45" s="13" t="n">
-        <x:v>46240.333333333336</x:v>
+        <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D45" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>未披露</x:v>
       </x:c>
       <x:c r="E45" s="12" t="str">
-        <x:v>B 轮</x:v>
+        <x:v>天使轮</x:v>
       </x:c>
       <x:c r="F45" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G45" s="14"/>
       <x:c r="H45" s="12" t="str">
-        <x:v>中国网</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I45" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E4%B8%BA%E5%85%89%E8%83%BD%E6%BA%90%20B%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202608/567448.shtml</x:v>
       </x:c>
       <x:c r="J45" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K45" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L45" s="12" t="str">
-        <x:v>西安为光能源科技有限公司聚焦固态变压器（SST）等新型电力电子装备及能源互联网解决方案。公司瞄准算力中心、电动交通、新型配网和储能等高功率密度场景，通过电能变换、控制和系统集成提升供配电效率与灵活性。</x:v>
+        <x:v>橡木果机器人专注通用具身操作，围绕触觉感知、操作基座模型和机器人执行能力构建底层技术栈。公司强调自下而上的“本能驱动”路线，目标是让机器人在真实物理环境中稳定完成操作任务。</x:v>
       </x:c>
       <x:c r="M45" s="12" t="str">
-        <x:v>https://www.weiguangenergy.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N45" s="12" t="str">
-        <x:v>服务热线：400-868-6988；商务邮箱（官网公开）：wangjuan0509@foxmail.com；地址：陕西省西安市高新区毕原二路3号先导院南区5-6号楼；公众号：WGenergy；在线留言：官网联系页。</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="12" t="str">
-        <x:v>飞捷科思</x:v>
+        <x:v>Noiz AI</x:v>
       </x:c>
       <x:c r="B46" s="12" t="str">
-        <x:v>半导体</x:v>
+        <x:v>AI 语音 / 视听内容生成</x:v>
       </x:c>
       <x:c r="C46" s="13" t="n">
-        <x:v>46240.333333333336</x:v>
+        <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D46" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E46" s="12" t="str">
-        <x:v>A1 轮</x:v>
+        <x:v>种子轮</x:v>
       </x:c>
       <x:c r="F46" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G46" s="14"/>
       <x:c r="H46" s="12" t="str">
-        <x:v>观点网</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I46" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E9%A3%9E%E6%8D%B7%E7%A7%91%E6%80%9D%20A1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202608/567447.shtml</x:v>
       </x:c>
       <x:c r="J46" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K46" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L46" s="12" t="str">
-        <x:v>飞捷科思以高精度实时物理仿真引擎为核心，研发面向具身智能和人形机器人的物理智能技术与产品。其能力重点在于让机器人在虚拟环境中完成动力学、接触和运动策略验证，以缩短从算法训练到真实机器部署的迭代周期。</x:v>
+        <x:v>Noiz AI 提供文本转语音、声音克隆和语音设计能力，面向内容创作、配音、本地化和开发者 API 场景。其产品强调情感控制、低延迟生成和多语言语音输出，服务全球化音频工作流。</x:v>
       </x:c>
       <x:c r="M46" s="12" t="str">
-        <x:v>https://fysics.net/</x:v>
+        <x:v>https://noiz.ai/</x:v>
       </x:c>
       <x:c r="N46" s="12" t="str">
-        <x:v>电话：021-60197571；商务邮箱：fysics@fysics.ai；官网联系页：https://fysics.net/contact.html。</x:v>
+        <x:v>邮箱：contact@noiz.ai；官网联系页：https://noiz.ai/。</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="12" t="str">
-        <x:v>蓝凌星通</x:v>
+        <x:v>飞声</x:v>
       </x:c>
       <x:c r="B47" s="12" t="str">
-        <x:v>卫星通信</x:v>
+        <x:v>AI 助听器 / 医疗器械</x:v>
       </x:c>
       <x:c r="C47" s="13" t="n">
-        <x:v>46240.333333333336</x:v>
+        <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D47" s="12" t="str">
         <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E47" s="12" t="str">
-        <x:v>股权融资</x:v>
+        <x:v>天使轮</x:v>
       </x:c>
       <x:c r="F47" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G47" s="14"/>
       <x:c r="H47" s="12" t="str">
-        <x:v>启迪之星</x:v>
+        <x:v>36氪</x:v>
       </x:c>
       <x:c r="I47" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E8%93%9D%E5%87%8C%E6%98%9F%E9%80%9A%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E9%A3%9E%E5%A3%B0%20AI%20%E5%8A%A9%E5%90%AC%E5%99%A8%20%E5%A4%A9%E4%BD%BF%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J47" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K47" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L47" s="12" t="str">
-        <x:v>蓝凌星通是蓝牙卫星系统服务商，利用低轨卫星为蓝牙终端提供低成本、低功耗的物联网连接和行业监测方案。其目标是把现有蓝牙终端延伸到传统地面网络覆盖不足的区域，服务户外、物流、资产追踪和行业监测等场景。</x:v>
+        <x:v>飞声专注 AI 助听器与听力辅助产品，结合声学处理、语音增强和智能交互能力改善听障场景的佩戴体验。公司面向消费级与医疗级场景推进产品化，强调清晰拾音、降噪和更自然的听觉补偿。</x:v>
       </x:c>
       <x:c r="M47" s="12" t="str">
-        <x:v>https://www.bluelinksatcom.com/</x:v>
+        <x:v>https://www.flysounds.cn/zh/</x:v>
       </x:c>
       <x:c r="N47" s="12" t="str">
-        <x:v>电话：400-8818-251；商务邮箱：market@bluelinksatcom.com。</x:v>
+        <x:v>电话：15828225541；商务邮箱：jory@flysounds.com；地址：深圳市龙华区龙华街道清湖社区大和路356号金鼎盛科创园A栋18楼。</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="12" t="str">
-        <x:v>RoboParty（萝博派对）</x:v>
+        <x:v>霍德生物</x:v>
       </x:c>
       <x:c r="B48" s="12" t="str">
-        <x:v>具身智能 / 人形机器人</x:v>
+        <x:v>细胞治疗 / 生物技术</x:v>
       </x:c>
       <x:c r="C48" s="13" t="n">
-        <x:v>46238.333333333336</x:v>
+        <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D48" s="12" t="str">
-        <x:v>近 5 亿元人民币</x:v>
+        <x:v>近 2 亿元人民币</x:v>
       </x:c>
       <x:c r="E48" s="12" t="str">
-        <x:v>天使++轮及 Pre-A 轮</x:v>
+        <x:v>C 轮首关</x:v>
       </x:c>
       <x:c r="F48" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G48" s="14"/>
       <x:c r="H48" s="12" t="str">
-        <x:v>快科技（新浪财经转载）</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I48" s="16" t="str">
-        <x:v>https://finance.sina.com.cn/tech/roll/2026-08-04/doc-inimchzp5821502.shtml</x:v>
+        <x:v>https://news.google.com/search?q=%E9%9C%8D%E5%BE%B7%E7%94%9F%E7%89%A9%20%E8%BF%91%202%20%E4%BA%BF%E5%85%83%20C%E8%BD%AE%20%E9%A6%96%E5%85%B3&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J48" s="15" t="n">
-        <x:v>46242.5</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K48" s="12" t="str">
-        <x:v>媒体交叉核验</x:v>
+        <x:v>媒体与公开工商信息交叉核验</x:v>
       </x:c>
       <x:c r="L48" s="12" t="str">
-        <x:v>RoboParty 专注低成本、高性能双足人形机器人研发，并通过全栈开源建设机器人开发生态。公司公开机器人结构、电气、训练和部署等技术资料，希望降低研究者与开发者进入人形机器人研发的门槛，并推动软硬件协同迭代。</x:v>
+        <x:v>霍德生物工程有限公司聚焦细胞治疗和再生医学相关技术与产品，围绕研发、工艺和临床转化推进管线建设。公司在公开页面中长期披露研发动态与产品进展，面向生物医药产业化需求。</x:v>
       </x:c>
       <x:c r="M48" s="12" t="str">
-        <x:v>https://roboparty.com/</x:v>
+        <x:v>https://www.hopstem.com/</x:v>
       </x:c>
       <x:c r="N48" s="12" t="str">
-        <x:v>商务邮箱：contact@roboparty.com；开源技术交流 QQ 群：1078670917；官方 GitHub：https://github.com/Roboparty。</x:v>
+        <x:v>电话：0571-88197776；邮箱：info@hopstem.com；官网联系页：https://www.hopstem.com/。</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="12" t="str">
-        <x:v>昉擎科技</x:v>
+        <x:v>可灵 AI</x:v>
       </x:c>
       <x:c r="B49" s="12" t="str">
-        <x:v>AI 算力芯片</x:v>
+        <x:v>AI 视频大模型</x:v>
       </x:c>
       <x:c r="C49" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46241.333333333336</x:v>
       </x:c>
       <x:c r="D49" s="12" t="str">
+        <x:v>近 30 亿美元</x:v>
+      </x:c>
+      <x:c r="E49" s="12" t="str">
         <x:v>未披露</x:v>
       </x:c>
-      <x:c r="E49" s="12" t="str">
-        <x:v>A1 轮</x:v>
-      </x:c>
       <x:c r="F49" s="12" t="str">
-        <x:v>CNY</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="G49" s="14"/>
       <x:c r="H49" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>新华网 / 经济参考报</x:v>
       </x:c>
       <x:c r="I49" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%98%89%E6%93%8E%E7%A7%91%E6%8A%80%20A1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://www.news.cn/tech/20260807/1605ef446e5045b7ba0ee55245ce731c/c.html</x:v>
       </x:c>
       <x:c r="J49" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46242.48541666667</x:v>
       </x:c>
       <x:c r="K49" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L49" s="12" t="str">
-        <x:v>昉擎科技是新一代智能计算系统企业，基于分离式架构和 4D Memory 理论，自主研发芯片、硬件系统与软件栈。公司重点解决 AI 计算系统的通用性、扩展性与工程化部署问题；本轮融资主要用于自研芯片和系统研发、规模化量产、软件生态建设及人才引进。</x:v>
+        <x:v>可灵 AI 是面向视频生成与创作的 AI 大模型产品，支持文本、图片等输入驱动的视频内容生成和编辑。产品服务广告创意、影视内容、社交媒体和商业化营销等场景，重点提升视频生成的一致性、可控性和创作效率。</x:v>
       </x:c>
       <x:c r="M49" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://klingai.com/</x:v>
       </x:c>
       <x:c r="N49" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>商务联系：官网联系页</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="12" t="str">
-        <x:v>协鑫光电</x:v>
+        <x:v>矩阵起源</x:v>
       </x:c>
       <x:c r="B50" s="12" t="str">
-        <x:v>钙钛矿光伏</x:v>
+        <x:v>企业级 AI 基础设施</x:v>
       </x:c>
       <x:c r="C50" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46240.333333333336</x:v>
       </x:c>
       <x:c r="D50" s="12" t="str">
-        <x:v>超 1 亿元人民币</x:v>
+        <x:v>超 1,000 万美元</x:v>
       </x:c>
       <x:c r="E50" s="12" t="str">
-        <x:v>D1 轮</x:v>
+        <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F50" s="12" t="str">
-        <x:v>CNY</x:v>
-      </x:c>
-      <x:c r="G50" s="14"/>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G50" s="14" t="n">
+        <x:v>7200</x:v>
+      </x:c>
       <x:c r="H50" s="12" t="str">
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I50" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%8D%8F%E9%91%AB%E5%85%89%E7%94%B5%20D1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E7%9F%A9%E9%98%B5%E8%B5%B7%E6%BA%90%20%E8%B6%85%E5%8D%83%E4%B8%87%E7%BE%8E%E5%85%83%20A%E8%BD%AE%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J50" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -2355,42 +2359,40 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L50" s="12" t="str">
-        <x:v>协鑫光电主要从事大面积钙钛矿光伏组件的研发、生产及商业化应用。公司围绕钙钛矿材料、组件制备、封装可靠性和量产工艺推进技术迭代，面向下一代高效率光伏组件及其应用市场。</x:v>
+        <x:v>矩阵起源专注 AI 原生数据基础设施，提供多模态数据处理、数据库与企业级 AI 数据底座产品及解决方案。其产品面向企业在结构化、非结构化和向量数据之间建立统一的数据管理与计算能力，为模型训练、知识检索和 AI 应用部署提供底层支撑。</x:v>
       </x:c>
       <x:c r="M50" s="12" t="str">
-        <x:v>https://www.gcl-perovskite.com/</x:v>
+        <x:v>https://matrixorigin.cn/</x:v>
       </x:c>
       <x:c r="N50" s="12" t="str">
-        <x:v>官网公开电话：86-0512-57562287；官网联系页：https://www.gcl-power.com/contact.html。</x:v>
+        <x:v>商务邮箱：contact@matrixorigin.cn。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="12" t="str">
-        <x:v>主动科技</x:v>
+        <x:v>为光能源</x:v>
       </x:c>
       <x:c r="B51" s="12" t="str">
-        <x:v>脑机接口</x:v>
+        <x:v>电力电子 / 固态变压器</x:v>
       </x:c>
       <x:c r="C51" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46240.333333333336</x:v>
       </x:c>
       <x:c r="D51" s="12" t="str">
-        <x:v>3.3 亿元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E51" s="12" t="str">
-        <x:v>天使轮</x:v>
+        <x:v>B 轮</x:v>
       </x:c>
       <x:c r="F51" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G51" s="14" t="n">
-        <x:v>33000</x:v>
-      </x:c>
+      <x:c r="G51" s="14"/>
       <x:c r="H51" s="12" t="str">
-        <x:v>观点网</x:v>
+        <x:v>中国网</x:v>
       </x:c>
       <x:c r="I51" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E4%B8%BB%E5%8A%A8%E7%A7%91%E6%8A%80%203.3%E4%BA%BF%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E4%B8%BA%E5%85%89%E8%83%BD%E6%BA%90%20B%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J51" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -2399,40 +2401,40 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L51" s="12" t="str">
-        <x:v>主动科技是一家侵入式脑机接口技术研发与产业化企业，核心产品为“天枢”运动脑机接口。公开报道显示，公司成立于 2026 年 2 月，正推进高通道脑机系统、微纳加工平台与临床试验，目标是推动侵入式脑机接口从实验室验证走向医疗器械产业化。</x:v>
+        <x:v>西安为光能源科技有限公司聚焦固态变压器（SST）等新型电力电子装备及能源互联网解决方案。公司瞄准算力中心、电动交通、新型配网和储能等高功率密度场景，通过电能变换、控制和系统集成提升供配电效率与灵活性。</x:v>
       </x:c>
       <x:c r="M51" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.weiguangenergy.com/</x:v>
       </x:c>
       <x:c r="N51" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>服务热线：400-868-6988；商务邮箱（官网公开）：wangjuan0509@foxmail.com；地址：陕西省西安市高新区毕原二路3号先导院南区5-6号楼；公众号：WGenergy；在线留言：官网联系页。</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="12" t="str">
-        <x:v>西湖心辰</x:v>
+        <x:v>飞捷科思</x:v>
       </x:c>
       <x:c r="B52" s="12" t="str">
-        <x:v>生成式 AI</x:v>
+        <x:v>半导体</x:v>
       </x:c>
       <x:c r="C52" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46240.333333333336</x:v>
       </x:c>
       <x:c r="D52" s="12" t="str">
         <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E52" s="12" t="str">
-        <x:v>B+ 轮</x:v>
+        <x:v>A1 轮</x:v>
       </x:c>
       <x:c r="F52" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G52" s="14"/>
       <x:c r="H52" s="12" t="str">
-        <x:v>澎湃新闻</x:v>
+        <x:v>观点网</x:v>
       </x:c>
       <x:c r="I52" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E8%A5%BF%E6%B9%96%E5%BF%83%E8%BE%B0%20B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E9%A3%9E%E6%8D%B7%E7%A7%91%E6%80%9D%20A1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J52" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -2441,40 +2443,40 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L52" s="12" t="str">
-        <x:v>西湖心辰是一家生成式 AI 公司，研发西湖大模型及面向创作与企业场景的 AI 原生应用。公司将大模型能力用于内容生成、智能交互和行业工作流，强调模型能力与实际产品体验、企业落地场景的结合。</x:v>
+        <x:v>飞捷科思以高精度实时物理仿真引擎为核心，研发面向具身智能和人形机器人的物理智能技术与产品。其能力重点在于让机器人在虚拟环境中完成动力学、接触和运动策略验证，以缩短从算法训练到真实机器部署的迭代周期。</x:v>
       </x:c>
       <x:c r="M52" s="12" t="str">
-        <x:v>https://xinchenai.com/</x:v>
+        <x:v>https://fysics.net/</x:v>
       </x:c>
       <x:c r="N52" s="12" t="str">
-        <x:v>电话：400-8126-618；邮箱：support@xinchenai.com；地址：浙江省杭州市西湖区智强路428号云创镓谷6号楼6楼604室。</x:v>
+        <x:v>电话：021-60197571；商务邮箱：fysics@fysics.ai；官网联系页：https://fysics.net/contact.html。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="12" t="str">
-        <x:v>璨辰科技</x:v>
+        <x:v>蓝凌星通</x:v>
       </x:c>
       <x:c r="B53" s="12" t="str">
-        <x:v>医疗 AI / 虚拟器官仿真</x:v>
+        <x:v>卫星通信</x:v>
       </x:c>
       <x:c r="C53" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46240.333333333336</x:v>
       </x:c>
       <x:c r="D53" s="12" t="str">
         <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E53" s="12" t="str">
-        <x:v>天使系列轮</x:v>
+        <x:v>股权融资</x:v>
       </x:c>
       <x:c r="F53" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G53" s="14"/>
       <x:c r="H53" s="12" t="str">
-        <x:v>雷峰网</x:v>
+        <x:v>启迪之星</x:v>
       </x:c>
       <x:c r="I53" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%92%A8%E8%BE%B0%E7%A7%91%E6%8A%80%20%E8%99%9A%E6%8B%9F%E5%99%A8%E5%AE%98%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E8%93%9D%E5%87%8C%E6%98%9F%E9%80%9A%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J53" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -2483,86 +2485,82 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L53" s="12" t="str">
-        <x:v>璨辰科技聚焦系统级虚拟器官时空动态演化模型研发，构建从分子、细胞、组织到器官的全尺度 AI 数字孪生平台。其方案服务于新药临床前评价、发育毒性评估与疾病机制研究，并通过“仿真—湿实验—临床前验证”的数据闭环提升模型的产业转化价值。</x:v>
+        <x:v>蓝凌星通是蓝牙卫星系统服务商，利用低轨卫星为蓝牙终端提供低成本、低功耗的物联网连接和行业监测方案。其目标是把现有蓝牙终端延伸到传统地面网络覆盖不足的区域，服务户外、物流、资产追踪和行业监测等场景。</x:v>
       </x:c>
       <x:c r="M53" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.bluelinksatcom.com/</x:v>
       </x:c>
       <x:c r="N53" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>电话：400-8818-251；商务邮箱：market@bluelinksatcom.com。</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="12" t="str">
-        <x:v>鸿鹄航空</x:v>
+        <x:v>RoboParty（萝博派对）</x:v>
       </x:c>
       <x:c r="B54" s="12" t="str">
-        <x:v>航空航天</x:v>
+        <x:v>具身智能 / 人形机器人</x:v>
       </x:c>
       <x:c r="C54" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46238.333333333336</x:v>
       </x:c>
       <x:c r="D54" s="12" t="str">
-        <x:v>7,000 万元人民币</x:v>
+        <x:v>近 5 亿元人民币</x:v>
       </x:c>
       <x:c r="E54" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>天使++轮及 Pre-A 轮</x:v>
       </x:c>
       <x:c r="F54" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G54" s="14" t="n">
-        <x:v>7000</x:v>
-      </x:c>
+      <x:c r="G54" s="14"/>
       <x:c r="H54" s="12" t="str">
-        <x:v>观点网</x:v>
+        <x:v>快科技（新浪财经转载）</x:v>
       </x:c>
       <x:c r="I54" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E9%B8%BF%E9%B9%84%E8%88%AA%E7%A9%BA%207000%E4%B8%87%20A%E8%BD%AE&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://finance.sina.com.cn/tech/roll/2026-08-04/doc-inimchzp5821502.shtml</x:v>
       </x:c>
       <x:c r="J54" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46242.5</x:v>
       </x:c>
       <x:c r="K54" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体交叉核验</x:v>
       </x:c>
       <x:c r="L54" s="12" t="str">
-        <x:v>青岛鸿鹄航空科技有限公司专注航空温控产品与服务，是海尔生物医疗控股子公司。公司围绕航空装备温度控制和相关系统服务开展产品研发，服务航空运行与专业运输等对环境控制要求较高的场景。</x:v>
+        <x:v>RoboParty 专注低成本、高性能双足人形机器人研发，并通过全栈开源建设机器人开发生态。公司公开机器人结构、电气、训练和部署等技术资料，希望降低研究者与开发者进入人形机器人研发的门槛，并推动软硬件协同迭代。</x:v>
       </x:c>
       <x:c r="M54" s="12" t="str">
-        <x:v>https://www.hbtempconaviation.com/</x:v>
+        <x:v>https://roboparty.com/</x:v>
       </x:c>
       <x:c r="N54" s="12" t="str">
-        <x:v>电话：+86-400-863-0863；邮箱：aviation@haierbiomedical.com；地址：青岛市高新区丰源路280号。</x:v>
+        <x:v>商务邮箱：contact@roboparty.com；开源技术交流 QQ 群：1078670917；官方 GitHub：https://github.com/Roboparty。</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
       <x:c r="A55" s="12" t="str">
-        <x:v>元育生物</x:v>
+        <x:v>昉擎科技</x:v>
       </x:c>
       <x:c r="B55" s="12" t="str">
-        <x:v>生物医药</x:v>
+        <x:v>AI 算力芯片</x:v>
       </x:c>
       <x:c r="C55" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D55" s="12" t="str">
-        <x:v>亿元人民币</x:v>
+        <x:v>未披露</x:v>
       </x:c>
       <x:c r="E55" s="12" t="str">
-        <x:v>A+ 轮</x:v>
+        <x:v>A1 轮</x:v>
       </x:c>
       <x:c r="F55" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G55" s="14" t="n">
-        <x:v>10000</x:v>
-      </x:c>
+      <x:c r="G55" s="14"/>
       <x:c r="H55" s="12" t="str">
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I55" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%85%83%E8%82%B2%E7%94%9F%E7%89%A9%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E6%98%89%E6%93%8E%E7%A7%91%E6%8A%80%20A1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J55" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -2571,252 +2569,256 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L55" s="12" t="str">
-        <x:v>元育生物是微藻生物合成企业，开发可持续微藻基原料并提供定制化应用解决方案。公司以微藻培养、代谢调控和生物制造为技术基础，探索在食品营养、功能原料、日化与绿色消费品等领域的产业化应用。</x:v>
+        <x:v>昉擎科技是新一代智能计算系统企业，基于分离式架构和 4D Memory 理论，自主研发芯片、硬件系统与软件栈。公司重点解决 AI 计算系统的通用性、扩展性与工程化部署问题；本轮融资主要用于自研芯片和系统研发、规模化量产、软件生态建设及人才引进。</x:v>
       </x:c>
       <x:c r="M55" s="12" t="str">
-        <x:v>https://www.protoga.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N55" s="12" t="str">
-        <x:v>珠海：0756-8699334；北京：010-67866793；海外 BD：bd@protoga.com；国内销售：sales@protoga.com；地址：广东省珠海市香洲区南屏镇科技工业园屏北一路30号1栋2楼。</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="12" t="str">
-        <x:v>幺正量子</x:v>
+        <x:v>协鑫光电</x:v>
       </x:c>
       <x:c r="B56" s="12" t="str">
-        <x:v>量子计算</x:v>
+        <x:v>钙钛矿光伏</x:v>
       </x:c>
       <x:c r="C56" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D56" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>超 1 亿元人民币</x:v>
       </x:c>
       <x:c r="E56" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>D1 轮</x:v>
       </x:c>
       <x:c r="F56" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G56" s="14"/>
       <x:c r="H56" s="12" t="str">
-        <x:v>大河财立方</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I56" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%B9%BA%E6%AD%A3%E9%87%8F%E5%AD%90%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E5%8D%8F%E9%91%AB%E5%85%89%E7%94%B5%20D1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J56" s="15" t="n">
-        <x:v>46242.479166666664</x:v>
+        <x:v>46241.479166666664</x:v>
       </x:c>
       <x:c r="K56" s="12" t="str">
-        <x:v>待官网交叉核验</x:v>
+        <x:v>已核验</x:v>
       </x:c>
       <x:c r="L56" s="12" t="str">
-        <x:v>幺正量子是一家离子阱量子计算企业，提供量子计算系统、设备器件、云服务和行业解决方案。公司围绕离子阱硬件、量子控制、算法与行业应用推进全栈研发，服务科研、教育和量子计算产业化需求。</x:v>
+        <x:v>协鑫光电主要从事大面积钙钛矿光伏组件的研发、生产及商业化应用。公司围绕钙钛矿材料、组件制备、封装可靠性和量产工艺推进技术迭代，面向下一代高效率光伏组件及其应用市场。</x:v>
       </x:c>
       <x:c r="M56" s="12" t="str">
-        <x:v>https://www.unitqc.com/</x:v>
+        <x:v>https://www.gcl-perovskite.com/</x:v>
       </x:c>
       <x:c r="N56" s="12" t="str">
-        <x:v>商务邮箱：business@unitqc.com；电话：15391985489；地址：安徽省合肥市高新区望江西路900号中安创谷科技园一期B1栋1-2层。</x:v>
+        <x:v>官网公开电话：86-0512-57562287；官网联系页：https://www.gcl-power.com/contact.html。</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="12" t="str">
-        <x:v>恺望数据</x:v>
+        <x:v>主动科技</x:v>
       </x:c>
       <x:c r="B57" s="12" t="str">
-        <x:v>AI 数据服务</x:v>
+        <x:v>脑机接口</x:v>
       </x:c>
       <x:c r="C57" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D57" s="12" t="str">
-        <x:v>逾亿元人民币</x:v>
+        <x:v>3.3 亿元人民币</x:v>
       </x:c>
       <x:c r="E57" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>天使轮</x:v>
       </x:c>
       <x:c r="F57" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G57" s="14"/>
+      <x:c r="G57" s="14" t="n">
+        <x:v>33000</x:v>
+      </x:c>
       <x:c r="H57" s="12" t="str">
-        <x:v>封面新闻</x:v>
+        <x:v>观点网</x:v>
       </x:c>
       <x:c r="I57" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%81%BA%E6%9C%9B%E6%95%B0%E6%8D%AE%20%E9%80%BE%E4%BA%BF%E5%85%83%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E4%B8%BB%E5%8A%A8%E7%A7%91%E6%8A%80%203.3%E4%BA%BF%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J57" s="15" t="n">
-        <x:v>46242.479166666664</x:v>
+        <x:v>46241.479166666664</x:v>
       </x:c>
       <x:c r="K57" s="12" t="str">
-        <x:v>待官网交叉核验</x:v>
+        <x:v>已核验</x:v>
       </x:c>
       <x:c r="L57" s="12" t="str">
-        <x:v>恺望数据为车企、自动驾驶及 AI 企业提供一站式数据解决方案和自动化数据生产能力。其服务覆盖数据采集、清洗、标注、质检和管理，重点支持自动驾驶、具身智能与大模型训练中的规模化高质量数据供给。</x:v>
+        <x:v>主动科技是一家侵入式脑机接口技术研发与产业化企业，核心产品为“天枢”运动脑机接口。公开报道显示，公司成立于 2026 年 2 月，正推进高通道脑机系统、微纳加工平台与临床试验，目标是推动侵入式脑机接口从实验室验证走向医疗器械产业化。</x:v>
       </x:c>
       <x:c r="M57" s="12" t="str">
-        <x:v>https://admin.d.konvery.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N57" s="12" t="str">
-        <x:v>官方产品平台：https://admin.d.konvery.com/；官网未公开完整商务电话或邮箱，可通过平台申请试用或联系。</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
       <x:c r="A58" s="12" t="str">
-        <x:v>求是光谱</x:v>
+        <x:v>西湖心辰</x:v>
       </x:c>
       <x:c r="B58" s="12" t="str">
-        <x:v>光谱检测</x:v>
+        <x:v>生成式 AI</x:v>
       </x:c>
       <x:c r="C58" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D58" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E58" s="12" t="str">
-        <x:v>B++ 轮</x:v>
+        <x:v>B+ 轮</x:v>
       </x:c>
       <x:c r="F58" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G58" s="14"/>
       <x:c r="H58" s="12" t="str">
-        <x:v>新浪财经</x:v>
+        <x:v>澎湃新闻</x:v>
       </x:c>
       <x:c r="I58" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%B1%82%E6%98%AF%E5%85%89%E8%B0%B1%20B%2B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E8%A5%BF%E6%B9%96%E5%BF%83%E8%BE%B0%20B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J58" s="15" t="n">
-        <x:v>46242.479166666664</x:v>
+        <x:v>46241.479166666664</x:v>
       </x:c>
       <x:c r="K58" s="12" t="str">
-        <x:v>待官网交叉核验</x:v>
+        <x:v>已核验</x:v>
       </x:c>
       <x:c r="L58" s="12" t="str">
-        <x:v>求是光谱从事多光谱成像芯片、光谱应用方案及光谱大数据研发，为智能终端、汽车电子、医疗和环境监测等场景提供产品与服务。公司将光谱感知能力嵌入硬件和软件方案，用于物质识别、成分分析和复杂环境下的智能检测。</x:v>
+        <x:v>西湖心辰是一家生成式 AI 公司，研发西湖大模型及面向创作与企业场景的 AI 原生应用。公司将大模型能力用于内容生成、智能交互和行业工作流，强调模型能力与实际产品体验、企业落地场景的结合。</x:v>
       </x:c>
       <x:c r="M58" s="12" t="str">
-        <x:v>https://www.qsspec.com/</x:v>
+        <x:v>https://xinchenai.com/</x:v>
       </x:c>
       <x:c r="N58" s="12" t="str">
-        <x:v>电话：0431-88882290；商务联系人：冯硕，18343025432，fengshuo@qsspec.com；展会公开邮箱：hanying@qsspec.com。</x:v>
+        <x:v>电话：400-8126-618；邮箱：support@xinchenai.com；地址：浙江省杭州市西湖区智强路428号云创镓谷6号楼6楼604室。</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="12" t="str">
-        <x:v>熵简科技</x:v>
+        <x:v>璨辰科技</x:v>
       </x:c>
       <x:c r="B59" s="12" t="str">
-        <x:v>企业软件 / 数据智能</x:v>
+        <x:v>医疗 AI / 虚拟器官仿真</x:v>
       </x:c>
       <x:c r="C59" s="13" t="n">
         <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D59" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E59" s="12" t="str">
-        <x:v>C 轮</x:v>
+        <x:v>天使系列轮</x:v>
       </x:c>
       <x:c r="F59" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G59" s="14"/>
       <x:c r="H59" s="12" t="str">
-        <x:v>新浪财经</x:v>
+        <x:v>雷峰网</x:v>
       </x:c>
       <x:c r="I59" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%86%B5%E7%AE%80%E7%A7%91%E6%8A%80%20C%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E7%92%A8%E8%BE%B0%E7%A7%91%E6%8A%80%20%E8%99%9A%E6%8B%9F%E5%99%A8%E5%AE%98%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J59" s="15" t="n">
-        <x:v>46242.479166666664</x:v>
+        <x:v>46241.479166666664</x:v>
       </x:c>
       <x:c r="K59" s="12" t="str">
-        <x:v>待官网交叉核验</x:v>
+        <x:v>已核验</x:v>
       </x:c>
       <x:c r="L59" s="12" t="str">
-        <x:v>熵简科技是面向金融资管行业的数字基础设施与数据智能服务商，提供另类数据、知识图谱和全域数据中台等能力。公司自主研发大数据分析引擎，帮助金融机构处理多源异构数据、构建标准化 API，并支持投研、风险管理和业务决策工作流。</x:v>
+        <x:v>璨辰科技聚焦系统级虚拟器官时空动态演化模型研发，构建从分子、细胞、组织到器官的全尺度 AI 数字孪生平台。其方案服务于新药临床前评价、发育毒性评估与疾病机制研究，并通过“仿真—湿实验—临床前验证”的数据闭环提升模型的产业转化价值。</x:v>
       </x:c>
       <x:c r="M59" s="12" t="str">
-        <x:v>https://www.valuesimplex.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N59" s="12" t="str">
-        <x:v>官网提供业务咨询入口；暂未检索到可交叉确认的公开商务电话或邮箱。</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
       <x:c r="A60" s="12" t="str">
-        <x:v>灏存科技</x:v>
+        <x:v>鸿鹄航空</x:v>
       </x:c>
       <x:c r="B60" s="12" t="str">
-        <x:v>硬科技</x:v>
+        <x:v>航空航天</x:v>
       </x:c>
       <x:c r="C60" s="13" t="n">
-        <x:v>46235.333333333336</x:v>
+        <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D60" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>7,000 万元人民币</x:v>
       </x:c>
       <x:c r="E60" s="12" t="str">
-        <x:v>A+ 轮</x:v>
+        <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F60" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G60" s="14"/>
+      <x:c r="G60" s="14" t="n">
+        <x:v>7000</x:v>
+      </x:c>
       <x:c r="H60" s="12" t="str">
-        <x:v>新浪财经</x:v>
+        <x:v>观点网</x:v>
       </x:c>
       <x:c r="I60" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%81%8F%E5%AD%98%E7%A7%91%E6%8A%80%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E9%B8%BF%E9%B9%84%E8%88%AA%E7%A9%BA%207000%E4%B8%87%20A%E8%BD%AE&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J60" s="15" t="n">
-        <x:v>46242.479166666664</x:v>
+        <x:v>46241.479166666664</x:v>
       </x:c>
       <x:c r="K60" s="12" t="str">
-        <x:v>待官网交叉核验</x:v>
+        <x:v>已核验</x:v>
       </x:c>
       <x:c r="L60" s="12" t="str">
-        <x:v>灏存科技从事人工智能穿戴型肢体动作识别软硬件技术研发，应用于 VR/AR/MR、电影工业和人形机器人运动感知场景。公司以穿戴式传感、人体动作捕捉和算法识别为核心，使虚拟交互、数字内容生产和机器人训练获得更细粒度的运动数据。</x:v>
+        <x:v>青岛鸿鹄航空科技有限公司专注航空温控产品与服务，是海尔生物医疗控股子公司。公司围绕航空装备温度控制和相关系统服务开展产品研发，服务航空运行与专业运输等对环境控制要求较高的场景。</x:v>
       </x:c>
       <x:c r="M60" s="12" t="str">
-        <x:v>https://www.hexacercle.com/</x:v>
+        <x:v>https://www.hbtempconaviation.com/</x:v>
       </x:c>
       <x:c r="N60" s="12" t="str">
-        <x:v>商务合作：+86 13349933396；邮箱：mike@hexacercle.com；武汉总部：武汉东湖高新区关东街道华工园三路湖北青创园4栋801。</x:v>
+        <x:v>电话：+86-400-863-0863；邮箱：aviation@haierbiomedical.com；地址：青岛市高新区丰源路280号。</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
       <x:c r="A61" s="12" t="str">
-        <x:v>月之暗面（Kimi）</x:v>
+        <x:v>元育生物</x:v>
       </x:c>
       <x:c r="B61" s="12" t="str">
-        <x:v>大模型</x:v>
+        <x:v>生物医药</x:v>
       </x:c>
       <x:c r="C61" s="13" t="n">
-        <x:v>46234.333333333336</x:v>
+        <x:v>46237.333333333336</x:v>
       </x:c>
       <x:c r="D61" s="12" t="str">
-        <x:v>超 35 亿美元</x:v>
+        <x:v>亿元人民币</x:v>
       </x:c>
       <x:c r="E61" s="12" t="str">
-        <x:v>F 轮</x:v>
+        <x:v>A+ 轮</x:v>
       </x:c>
       <x:c r="F61" s="12" t="str">
-        <x:v>USD</x:v>
+        <x:v>CNY</x:v>
       </x:c>
       <x:c r="G61" s="14" t="n">
-        <x:v>2520000</x:v>
+        <x:v>10000</x:v>
       </x:c>
       <x:c r="H61" s="12" t="str">
-        <x:v>创业邦</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I61" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%9C%88%E4%B9%8B%E6%9A%97%E9%9D%A2%20F%E8%BD%AE%2035%E4%BA%BF%E7%BE%8E%E5%85%83&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E5%85%83%E8%82%B2%E7%94%9F%E7%89%A9%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J61" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -2825,12 +2827,266 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L61" s="12" t="str">
+        <x:v>元育生物是微藻生物合成企业，开发可持续微藻基原料并提供定制化应用解决方案。公司以微藻培养、代谢调控和生物制造为技术基础，探索在食品营养、功能原料、日化与绿色消费品等领域的产业化应用。</x:v>
+      </x:c>
+      <x:c r="M61" s="12" t="str">
+        <x:v>https://www.protoga.com/</x:v>
+      </x:c>
+      <x:c r="N61" s="12" t="str">
+        <x:v>珠海：0756-8699334；北京：010-67866793；海外 BD：bd@protoga.com；国内销售：sales@protoga.com；地址：广东省珠海市香洲区南屏镇科技工业园屏北一路30号1栋2楼。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="15" hidden="0" customHeight="1">
+      <x:c r="A62" s="12" t="str">
+        <x:v>幺正量子</x:v>
+      </x:c>
+      <x:c r="B62" s="12" t="str">
+        <x:v>量子计算</x:v>
+      </x:c>
+      <x:c r="C62" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D62" s="12" t="str">
+        <x:v>数亿元人民币</x:v>
+      </x:c>
+      <x:c r="E62" s="12" t="str">
+        <x:v>A 轮</x:v>
+      </x:c>
+      <x:c r="F62" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G62" s="14"/>
+      <x:c r="H62" s="12" t="str">
+        <x:v>大河财立方</x:v>
+      </x:c>
+      <x:c r="I62" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E5%B9%BA%E6%AD%A3%E9%87%8F%E5%AD%90%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J62" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K62" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L62" s="12" t="str">
+        <x:v>幺正量子是一家离子阱量子计算企业，提供量子计算系统、设备器件、云服务和行业解决方案。公司围绕离子阱硬件、量子控制、算法与行业应用推进全栈研发，服务科研、教育和量子计算产业化需求。</x:v>
+      </x:c>
+      <x:c r="M62" s="12" t="str">
+        <x:v>https://www.unitqc.com/</x:v>
+      </x:c>
+      <x:c r="N62" s="12" t="str">
+        <x:v>商务邮箱：business@unitqc.com；电话：15391985489；地址：安徽省合肥市高新区望江西路900号中安创谷科技园一期B1栋1-2层。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="15" hidden="0" customHeight="1">
+      <x:c r="A63" s="12" t="str">
+        <x:v>恺望数据</x:v>
+      </x:c>
+      <x:c r="B63" s="12" t="str">
+        <x:v>AI 数据服务</x:v>
+      </x:c>
+      <x:c r="C63" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D63" s="12" t="str">
+        <x:v>逾亿元人民币</x:v>
+      </x:c>
+      <x:c r="E63" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="F63" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G63" s="14"/>
+      <x:c r="H63" s="12" t="str">
+        <x:v>封面新闻</x:v>
+      </x:c>
+      <x:c r="I63" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E6%81%BA%E6%9C%9B%E6%95%B0%E6%8D%AE%20%E9%80%BE%E4%BA%BF%E5%85%83%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J63" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K63" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L63" s="12" t="str">
+        <x:v>恺望数据为车企、自动驾驶及 AI 企业提供一站式数据解决方案和自动化数据生产能力。其服务覆盖数据采集、清洗、标注、质检和管理，重点支持自动驾驶、具身智能与大模型训练中的规模化高质量数据供给。</x:v>
+      </x:c>
+      <x:c r="M63" s="12" t="str">
+        <x:v>https://admin.d.konvery.com/</x:v>
+      </x:c>
+      <x:c r="N63" s="12" t="str">
+        <x:v>官方产品平台：https://admin.d.konvery.com/；官网未公开完整商务电话或邮箱，可通过平台申请试用或联系。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="15" hidden="0" customHeight="1">
+      <x:c r="A64" s="12" t="str">
+        <x:v>求是光谱</x:v>
+      </x:c>
+      <x:c r="B64" s="12" t="str">
+        <x:v>光谱检测</x:v>
+      </x:c>
+      <x:c r="C64" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D64" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="E64" s="12" t="str">
+        <x:v>B++ 轮</x:v>
+      </x:c>
+      <x:c r="F64" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G64" s="14"/>
+      <x:c r="H64" s="12" t="str">
+        <x:v>新浪财经</x:v>
+      </x:c>
+      <x:c r="I64" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E6%B1%82%E6%98%AF%E5%85%89%E8%B0%B1%20B%2B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J64" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K64" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L64" s="12" t="str">
+        <x:v>求是光谱从事多光谱成像芯片、光谱应用方案及光谱大数据研发，为智能终端、汽车电子、医疗和环境监测等场景提供产品与服务。公司将光谱感知能力嵌入硬件和软件方案，用于物质识别、成分分析和复杂环境下的智能检测。</x:v>
+      </x:c>
+      <x:c r="M64" s="12" t="str">
+        <x:v>https://www.qsspec.com/</x:v>
+      </x:c>
+      <x:c r="N64" s="12" t="str">
+        <x:v>电话：0431-88882290；商务联系人：冯硕，18343025432，fengshuo@qsspec.com；展会公开邮箱：hanying@qsspec.com。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="15" hidden="0" customHeight="1">
+      <x:c r="A65" s="12" t="str">
+        <x:v>熵简科技</x:v>
+      </x:c>
+      <x:c r="B65" s="12" t="str">
+        <x:v>企业软件 / 数据智能</x:v>
+      </x:c>
+      <x:c r="C65" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D65" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="E65" s="12" t="str">
+        <x:v>C 轮</x:v>
+      </x:c>
+      <x:c r="F65" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G65" s="14"/>
+      <x:c r="H65" s="12" t="str">
+        <x:v>新浪财经</x:v>
+      </x:c>
+      <x:c r="I65" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E7%86%B5%E7%AE%80%E7%A7%91%E6%8A%80%20C%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J65" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K65" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L65" s="12" t="str">
+        <x:v>熵简科技是面向金融资管行业的数字基础设施与数据智能服务商，提供另类数据、知识图谱和全域数据中台等能力。公司自主研发大数据分析引擎，帮助金融机构处理多源异构数据、构建标准化 API，并支持投研、风险管理和业务决策工作流。</x:v>
+      </x:c>
+      <x:c r="M65" s="12" t="str">
+        <x:v>https://www.valuesimplex.com/</x:v>
+      </x:c>
+      <x:c r="N65" s="12" t="str">
+        <x:v>官网提供业务咨询入口；暂未检索到可交叉确认的公开商务电话或邮箱。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="15" hidden="0" customHeight="1">
+      <x:c r="A66" s="12" t="str">
+        <x:v>灏存科技</x:v>
+      </x:c>
+      <x:c r="B66" s="12" t="str">
+        <x:v>硬科技</x:v>
+      </x:c>
+      <x:c r="C66" s="13" t="n">
+        <x:v>46235.333333333336</x:v>
+      </x:c>
+      <x:c r="D66" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="E66" s="12" t="str">
+        <x:v>A+ 轮</x:v>
+      </x:c>
+      <x:c r="F66" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G66" s="14"/>
+      <x:c r="H66" s="12" t="str">
+        <x:v>新浪财经</x:v>
+      </x:c>
+      <x:c r="I66" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E7%81%8F%E5%AD%98%E7%A7%91%E6%8A%80%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J66" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K66" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L66" s="12" t="str">
+        <x:v>灏存科技从事人工智能穿戴型肢体动作识别软硬件技术研发，应用于 VR/AR/MR、电影工业和人形机器人运动感知场景。公司以穿戴式传感、人体动作捕捉和算法识别为核心，使虚拟交互、数字内容生产和机器人训练获得更细粒度的运动数据。</x:v>
+      </x:c>
+      <x:c r="M66" s="12" t="str">
+        <x:v>https://www.hexacercle.com/</x:v>
+      </x:c>
+      <x:c r="N66" s="12" t="str">
+        <x:v>商务合作：+86 13349933396；邮箱：mike@hexacercle.com；武汉总部：武汉东湖高新区关东街道华工园三路湖北青创园4栋801。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="15" hidden="0" customHeight="1">
+      <x:c r="A67" s="12" t="str">
+        <x:v>月之暗面（Kimi）</x:v>
+      </x:c>
+      <x:c r="B67" s="12" t="str">
+        <x:v>大模型</x:v>
+      </x:c>
+      <x:c r="C67" s="13" t="n">
+        <x:v>46234.333333333336</x:v>
+      </x:c>
+      <x:c r="D67" s="12" t="str">
+        <x:v>超 35 亿美元</x:v>
+      </x:c>
+      <x:c r="E67" s="12" t="str">
+        <x:v>F 轮</x:v>
+      </x:c>
+      <x:c r="F67" s="12" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G67" s="14" t="n">
+        <x:v>2520000</x:v>
+      </x:c>
+      <x:c r="H67" s="12" t="str">
+        <x:v>创业邦</x:v>
+      </x:c>
+      <x:c r="I67" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E6%9C%88%E4%B9%8B%E6%9A%97%E9%9D%A2%20F%E8%BD%AE%2035%E4%BA%BF%E7%BE%8E%E5%85%83&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J67" s="15" t="n">
+        <x:v>46241.479166666664</x:v>
+      </x:c>
+      <x:c r="K67" s="12" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="L67" s="12" t="str">
         <x:v>月之暗面是一家大模型创业公司，推出 Kimi 等面向个人与企业的 AI 产品。其产品以长上下文理解、资料阅读、信息整理和多轮对话为主要能力，覆盖个人效率工具与企业级 AI 应用需求。</x:v>
       </x:c>
-      <x:c r="M61" s="12" t="str">
+      <x:c r="M67" s="12" t="str">
         <x:v>https://www.moonshot.cn/</x:v>
       </x:c>
-      <x:c r="N61" s="12" t="str">
+      <x:c r="N67" s="12" t="str">
         <x:v>产品/售后：support@moonshot.cn；媒体：pr@kimi.com；投资者联系：ir@kimi.com；企业微信客服：微信公众号「月之暗面Kimi」菜单“联系我们”。</x:v>
       </x:c>
     </x:row>
@@ -3284,10 +3540,10 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="18" t="n">
-        <x:v>46272.4316646875</x:v>
+        <x:v>46283.20244277778</x:v>
       </x:c>
       <x:c r="B2" t="n">
-        <x:v>57</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C2" t="n">
         <x:v>7</x:v>

</xml_diff>